<commit_message>
Binary Search Tree added
</commit_message>
<xml_diff>
--- a/FINAL450.xlsx
+++ b/FINAL450.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="532">
   <si>
     <t xml:space="preserve">YES(Iterative &amp; recursive)</t>
   </si>
@@ -862,15 +862,24 @@
     <t xml:space="preserve">Fina a value in a BST</t>
   </si>
   <si>
+    <t xml:space="preserve">y(search and insert leaf)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Deletion of a node in a BST</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(recursive and iterative)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Find min and max value in a BST</t>
   </si>
   <si>
     <t xml:space="preserve">Find inorder successor and inorder predecessor in a BST</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see condtion if key not present in tree)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Check if a tree is a BST or not </t>
   </si>
   <si>
@@ -883,6 +892,9 @@
     <t xml:space="preserve">Construct BST from preorder traversal</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Check modified recursion (using range))</t>
+  </si>
+  <si>
     <t xml:space="preserve">Convert Binary tree into BST</t>
   </si>
   <si>
@@ -898,12 +910,18 @@
     <t xml:space="preserve">Find Kth smallest element in a BST</t>
   </si>
   <si>
+    <t xml:space="preserve">y(similar to previous)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Count pairs from 2 BST whose sum is equal to given value "X"</t>
   </si>
   <si>
     <t xml:space="preserve">Find the median of BST in O(n) time and O(1) space</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(MORRIS INORDER TRAVERSAL)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Count BST ndoes that lie in a given range</t>
   </si>
   <si>
@@ -920,6 +938,9 @@
   </si>
   <si>
     <t xml:space="preserve">Largest BST in a Binary Tree [ V.V.V.V.V IMP ]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES(postorder return info of each subtree)</t>
   </si>
   <si>
     <t xml:space="preserve">Flatten BST to sorted list</t>
@@ -1907,11 +1928,12 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C481"/>
-  <sheetFormatPr defaultColWidth="11.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="111.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="37.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="4" style="0" width="11.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4161,7 +4183,7 @@
         <v>269</v>
       </c>
       <c r="C214" s="6" t="s">
-        <v>119</v>
+        <v>270</v>
       </c>
     </row>
     <row r="215" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4169,21 +4191,21 @@
         <v>268</v>
       </c>
       <c r="B215" s="8" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C215" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="216" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="216" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B216" s="8" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C216" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="217" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4191,10 +4213,10 @@
         <v>268</v>
       </c>
       <c r="B217" s="8" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C217" s="6" t="s">
-        <v>119</v>
+        <v>275</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4202,10 +4224,10 @@
         <v>268</v>
       </c>
       <c r="B218" s="8" t="s">
-        <v>273</v>
-      </c>
-      <c r="C218" s="6" t="s">
-        <v>119</v>
+        <v>276</v>
+      </c>
+      <c r="C218" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4213,10 +4235,10 @@
         <v>268</v>
       </c>
       <c r="B219" s="8" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C219" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4224,10 +4246,10 @@
         <v>268</v>
       </c>
       <c r="B220" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C220" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="221" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4235,10 +4257,10 @@
         <v>268</v>
       </c>
       <c r="B221" s="8" t="s">
-        <v>276</v>
-      </c>
-      <c r="C221" s="6" t="s">
-        <v>119</v>
+        <v>279</v>
+      </c>
+      <c r="C221" s="9" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4246,21 +4268,21 @@
         <v>268</v>
       </c>
       <c r="B222" s="8" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C222" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="223" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="223" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B223" s="8" t="s">
-        <v>278</v>
-      </c>
-      <c r="C223" s="6" t="s">
-        <v>119</v>
+        <v>282</v>
+      </c>
+      <c r="C223" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4268,21 +4290,21 @@
         <v>268</v>
       </c>
       <c r="B224" s="8" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C224" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="225" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="225" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B225" s="8" t="s">
-        <v>280</v>
-      </c>
-      <c r="C225" s="6" t="s">
-        <v>119</v>
+        <v>284</v>
+      </c>
+      <c r="C225" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="226" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4290,10 +4312,10 @@
         <v>268</v>
       </c>
       <c r="B226" s="8" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="C226" s="6" t="s">
-        <v>119</v>
+        <v>286</v>
       </c>
     </row>
     <row r="227" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4301,21 +4323,21 @@
         <v>268</v>
       </c>
       <c r="B227" s="8" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C227" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="228" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="228" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B228" s="8" t="s">
-        <v>283</v>
-      </c>
-      <c r="C228" s="6" t="s">
-        <v>119</v>
+        <v>288</v>
+      </c>
+      <c r="C228" s="9" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="229" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4323,10 +4345,10 @@
         <v>268</v>
       </c>
       <c r="B229" s="8" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C229" s="6" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="230" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4334,21 +4356,21 @@
         <v>268</v>
       </c>
       <c r="B230" s="8" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="C230" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="231" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="231" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B231" s="8" t="s">
-        <v>286</v>
-      </c>
-      <c r="C231" s="6" t="s">
-        <v>119</v>
+        <v>292</v>
+      </c>
+      <c r="C231" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="232" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4356,10 +4378,10 @@
         <v>268</v>
       </c>
       <c r="B232" s="8" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C232" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="233" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4367,32 +4389,32 @@
         <v>268</v>
       </c>
       <c r="B233" s="8" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C233" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="234" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="234" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B234" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="C234" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="235" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>295</v>
+      </c>
+      <c r="C234" s="9" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="235" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="7" t="s">
         <v>268</v>
       </c>
       <c r="B235" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="C235" s="6" t="s">
-        <v>119</v>
+        <v>297</v>
+      </c>
+      <c r="C235" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="236" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4408,10 +4430,10 @@
     </row>
     <row r="238" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B238" s="8" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="C238" s="6" t="s">
         <v>119</v>
@@ -4419,10 +4441,10 @@
     </row>
     <row r="239" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B239" s="8" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="C239" s="6" t="s">
         <v>119</v>
@@ -4430,10 +4452,10 @@
     </row>
     <row r="240" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B240" s="8" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="C240" s="6" t="s">
         <v>119</v>
@@ -4441,10 +4463,10 @@
     </row>
     <row r="241" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A241" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B241" s="8" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="C241" s="6" t="s">
         <v>119</v>
@@ -4452,10 +4474,10 @@
     </row>
     <row r="242" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A242" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B242" s="8" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="C242" s="6" t="s">
         <v>119</v>
@@ -4463,10 +4485,10 @@
     </row>
     <row r="243" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A243" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B243" s="8" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="C243" s="6" t="s">
         <v>119</v>
@@ -4474,10 +4496,10 @@
     </row>
     <row r="244" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A244" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B244" s="8" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="C244" s="6" t="s">
         <v>119</v>
@@ -4485,10 +4507,10 @@
     </row>
     <row r="245" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A245" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B245" s="8" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="C245" s="6" t="s">
         <v>119</v>
@@ -4496,10 +4518,10 @@
     </row>
     <row r="246" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A246" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B246" s="8" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C246" s="6" t="s">
         <v>119</v>
@@ -4507,10 +4529,10 @@
     </row>
     <row r="247" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A247" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B247" s="8" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="C247" s="6" t="s">
         <v>119</v>
@@ -4518,10 +4540,10 @@
     </row>
     <row r="248" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A248" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B248" s="8" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="C248" s="6" t="s">
         <v>119</v>
@@ -4529,10 +4551,10 @@
     </row>
     <row r="249" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B249" s="8" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C249" s="6" t="s">
         <v>119</v>
@@ -4540,10 +4562,10 @@
     </row>
     <row r="250" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B250" s="8" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C250" s="6" t="s">
         <v>119</v>
@@ -4551,10 +4573,10 @@
     </row>
     <row r="251" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A251" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B251" s="8" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="C251" s="6" t="s">
         <v>119</v>
@@ -4562,10 +4584,10 @@
     </row>
     <row r="252" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A252" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B252" s="8" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="C252" s="6" t="s">
         <v>119</v>
@@ -4573,10 +4595,10 @@
     </row>
     <row r="253" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A253" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B253" s="8" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="C253" s="6" t="s">
         <v>119</v>
@@ -4584,10 +4606,10 @@
     </row>
     <row r="254" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A254" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B254" s="8" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="C254" s="6" t="s">
         <v>119</v>
@@ -4595,10 +4617,10 @@
     </row>
     <row r="255" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A255" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B255" s="8" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C255" s="6" t="s">
         <v>119</v>
@@ -4606,10 +4628,10 @@
     </row>
     <row r="256" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A256" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B256" s="8" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C256" s="6" t="s">
         <v>119</v>
@@ -4617,10 +4639,10 @@
     </row>
     <row r="257" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A257" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B257" s="8" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C257" s="6" t="s">
         <v>119</v>
@@ -4628,10 +4650,10 @@
     </row>
     <row r="258" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A258" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B258" s="8" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="C258" s="6" t="s">
         <v>119</v>
@@ -4639,10 +4661,10 @@
     </row>
     <row r="259" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B259" s="8" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C259" s="6" t="s">
         <v>119</v>
@@ -4650,10 +4672,10 @@
     </row>
     <row r="260" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A260" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B260" s="8" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="C260" s="6" t="s">
         <v>119</v>
@@ -4661,10 +4683,10 @@
     </row>
     <row r="261" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B261" s="8" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="C261" s="6" t="s">
         <v>119</v>
@@ -4672,10 +4694,10 @@
     </row>
     <row r="262" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A262" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B262" s="8" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C262" s="6" t="s">
         <v>119</v>
@@ -4683,10 +4705,10 @@
     </row>
     <row r="263" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B263" s="8" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="C263" s="6" t="s">
         <v>119</v>
@@ -4694,10 +4716,10 @@
     </row>
     <row r="264" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B264" s="8" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="C264" s="6" t="s">
         <v>119</v>
@@ -4705,10 +4727,10 @@
     </row>
     <row r="265" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B265" s="8" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="C265" s="6" t="s">
         <v>119</v>
@@ -4716,10 +4738,10 @@
     </row>
     <row r="266" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A266" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B266" s="8" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="C266" s="6" t="s">
         <v>119</v>
@@ -4727,10 +4749,10 @@
     </row>
     <row r="267" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A267" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B267" s="8" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="C267" s="6" t="s">
         <v>119</v>
@@ -4738,10 +4760,10 @@
     </row>
     <row r="268" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B268" s="8" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C268" s="6" t="s">
         <v>119</v>
@@ -4749,10 +4771,10 @@
     </row>
     <row r="269" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B269" s="8" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="C269" s="6" t="s">
         <v>119</v>
@@ -4760,10 +4782,10 @@
     </row>
     <row r="270" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B270" s="8" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="C270" s="6" t="s">
         <v>119</v>
@@ -4771,7 +4793,7 @@
     </row>
     <row r="271" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B271" s="8" t="s">
         <v>120</v>
@@ -4782,10 +4804,10 @@
     </row>
     <row r="272" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="7" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B272" s="8" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="C272" s="6" t="s">
         <v>119</v>
@@ -4797,17 +4819,17 @@
     </row>
     <row r="274" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A274" s="0" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B274" s="10"/>
       <c r="C274" s="6"/>
     </row>
     <row r="275" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B275" s="8" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="C275" s="6" t="s">
         <v>119</v>
@@ -4815,10 +4837,10 @@
     </row>
     <row r="276" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B276" s="8" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="C276" s="6" t="s">
         <v>119</v>
@@ -4826,10 +4848,10 @@
     </row>
     <row r="277" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A277" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B277" s="8" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="C277" s="6" t="s">
         <v>119</v>
@@ -4837,10 +4859,10 @@
     </row>
     <row r="278" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B278" s="8" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="C278" s="6" t="s">
         <v>119</v>
@@ -4848,10 +4870,10 @@
     </row>
     <row r="279" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B279" s="8" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="C279" s="6" t="s">
         <v>119</v>
@@ -4859,10 +4881,10 @@
     </row>
     <row r="280" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B280" s="8" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="C280" s="6" t="s">
         <v>119</v>
@@ -4870,10 +4892,10 @@
     </row>
     <row r="281" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B281" s="8" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="C281" s="6" t="s">
         <v>119</v>
@@ -4881,10 +4903,10 @@
     </row>
     <row r="282" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A282" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B282" s="8" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="C282" s="6" t="s">
         <v>119</v>
@@ -4892,10 +4914,10 @@
     </row>
     <row r="283" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B283" s="8" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="C283" s="6" t="s">
         <v>119</v>
@@ -4903,10 +4925,10 @@
     </row>
     <row r="284" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B284" s="8" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="C284" s="6" t="s">
         <v>119</v>
@@ -4914,10 +4936,10 @@
     </row>
     <row r="285" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B285" s="8" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="C285" s="6" t="s">
         <v>119</v>
@@ -4925,10 +4947,10 @@
     </row>
     <row r="286" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B286" s="8" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="C286" s="6" t="s">
         <v>119</v>
@@ -4936,10 +4958,10 @@
     </row>
     <row r="287" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B287" s="8" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="C287" s="6" t="s">
         <v>119</v>
@@ -4947,10 +4969,10 @@
     </row>
     <row r="288" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B288" s="8" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="C288" s="6" t="s">
         <v>119</v>
@@ -4958,10 +4980,10 @@
     </row>
     <row r="289" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B289" s="8" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="C289" s="6" t="s">
         <v>119</v>
@@ -4969,10 +4991,10 @@
     </row>
     <row r="290" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A290" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B290" s="8" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="C290" s="6" t="s">
         <v>119</v>
@@ -4980,10 +5002,10 @@
     </row>
     <row r="291" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B291" s="8" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="C291" s="6" t="s">
         <v>119</v>
@@ -4991,10 +5013,10 @@
     </row>
     <row r="292" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B292" s="8" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="C292" s="6" t="s">
         <v>119</v>
@@ -5002,10 +5024,10 @@
     </row>
     <row r="293" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="7" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B293" s="8" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C293" s="6" t="s">
         <v>119</v>
@@ -5024,10 +5046,10 @@
     </row>
     <row r="296" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A296" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B296" s="8" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="C296" s="6" t="s">
         <v>119</v>
@@ -5035,10 +5057,10 @@
     </row>
     <row r="297" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A297" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B297" s="8" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="C297" s="6" t="s">
         <v>119</v>
@@ -5046,10 +5068,10 @@
     </row>
     <row r="298" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A298" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B298" s="8" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="C298" s="6" t="s">
         <v>119</v>
@@ -5057,10 +5079,10 @@
     </row>
     <row r="299" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B299" s="8" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="C299" s="6" t="s">
         <v>119</v>
@@ -5068,10 +5090,10 @@
     </row>
     <row r="300" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A300" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B300" s="8" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="C300" s="6" t="s">
         <v>119</v>
@@ -5079,10 +5101,10 @@
     </row>
     <row r="301" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A301" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B301" s="8" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="C301" s="6" t="s">
         <v>119</v>
@@ -5090,10 +5112,10 @@
     </row>
     <row r="302" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A302" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B302" s="8" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="C302" s="6" t="s">
         <v>119</v>
@@ -5101,10 +5123,10 @@
     </row>
     <row r="303" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A303" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B303" s="8" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="C303" s="6" t="s">
         <v>119</v>
@@ -5112,10 +5134,10 @@
     </row>
     <row r="304" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A304" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B304" s="8" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C304" s="6" t="s">
         <v>119</v>
@@ -5123,10 +5145,10 @@
     </row>
     <row r="305" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A305" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B305" s="8" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="C305" s="6" t="s">
         <v>119</v>
@@ -5134,10 +5156,10 @@
     </row>
     <row r="306" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B306" s="8" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="C306" s="6" t="s">
         <v>119</v>
@@ -5145,10 +5167,10 @@
     </row>
     <row r="307" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A307" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B307" s="8" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C307" s="6" t="s">
         <v>119</v>
@@ -5156,10 +5178,10 @@
     </row>
     <row r="308" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B308" s="8" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="C308" s="6" t="s">
         <v>119</v>
@@ -5167,10 +5189,10 @@
     </row>
     <row r="309" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A309" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B309" s="12" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="C309" s="6" t="s">
         <v>119</v>
@@ -5178,10 +5200,10 @@
     </row>
     <row r="310" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A310" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B310" s="8" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C310" s="6" t="s">
         <v>119</v>
@@ -5189,10 +5211,10 @@
     </row>
     <row r="311" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A311" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B311" s="8" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="C311" s="6" t="s">
         <v>119</v>
@@ -5200,10 +5222,10 @@
     </row>
     <row r="312" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B312" s="8" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="C312" s="6" t="s">
         <v>119</v>
@@ -5211,10 +5233,10 @@
     </row>
     <row r="313" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B313" s="8" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="C313" s="6" t="s">
         <v>119</v>
@@ -5222,10 +5244,10 @@
     </row>
     <row r="314" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B314" s="8" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="C314" s="6" t="s">
         <v>119</v>
@@ -5233,10 +5255,10 @@
     </row>
     <row r="315" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A315" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B315" s="8" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="C315" s="6" t="s">
         <v>119</v>
@@ -5244,10 +5266,10 @@
     </row>
     <row r="316" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A316" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B316" s="8" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="C316" s="6" t="s">
         <v>119</v>
@@ -5255,10 +5277,10 @@
     </row>
     <row r="317" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A317" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B317" s="8" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="C317" s="6" t="s">
         <v>119</v>
@@ -5266,10 +5288,10 @@
     </row>
     <row r="318" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B318" s="8" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="C318" s="6" t="s">
         <v>119</v>
@@ -5277,10 +5299,10 @@
     </row>
     <row r="319" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A319" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B319" s="8" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="C319" s="6" t="s">
         <v>119</v>
@@ -5288,10 +5310,10 @@
     </row>
     <row r="320" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B320" s="8" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="C320" s="6" t="s">
         <v>119</v>
@@ -5299,10 +5321,10 @@
     </row>
     <row r="321" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B321" s="8" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="C321" s="6" t="s">
         <v>119</v>
@@ -5310,10 +5332,10 @@
     </row>
     <row r="322" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A322" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B322" s="8" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="C322" s="6" t="s">
         <v>119</v>
@@ -5321,10 +5343,10 @@
     </row>
     <row r="323" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B323" s="8" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="C323" s="6" t="s">
         <v>119</v>
@@ -5332,10 +5354,10 @@
     </row>
     <row r="324" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B324" s="8" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="C324" s="6" t="s">
         <v>119</v>
@@ -5343,10 +5365,10 @@
     </row>
     <row r="325" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A325" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B325" s="8" t="s">
-        <v>376</v>
+        <v>383</v>
       </c>
       <c r="C325" s="6" t="s">
         <v>119</v>
@@ -5354,10 +5376,10 @@
     </row>
     <row r="326" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B326" s="8" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="C326" s="6" t="s">
         <v>119</v>
@@ -5365,10 +5387,10 @@
     </row>
     <row r="327" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A327" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B327" s="8" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C327" s="6" t="s">
         <v>119</v>
@@ -5376,10 +5398,10 @@
     </row>
     <row r="328" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A328" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B328" s="8" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="C328" s="6" t="s">
         <v>119</v>
@@ -5387,10 +5409,10 @@
     </row>
     <row r="329" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A329" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B329" s="8" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="C329" s="6" t="s">
         <v>119</v>
@@ -5398,10 +5420,10 @@
     </row>
     <row r="330" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A330" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B330" s="8" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="C330" s="6" t="s">
         <v>119</v>
@@ -5409,10 +5431,10 @@
     </row>
     <row r="331" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B331" s="8" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="C331" s="6" t="s">
         <v>119</v>
@@ -5420,10 +5442,10 @@
     </row>
     <row r="332" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A332" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B332" s="8" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="C332" s="6" t="s">
         <v>119</v>
@@ -5431,10 +5453,10 @@
     </row>
     <row r="333" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A333" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B333" s="8" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="C333" s="6" t="s">
         <v>119</v>
@@ -5453,10 +5475,10 @@
     </row>
     <row r="336" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B336" s="8" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="C336" s="6" t="s">
         <v>119</v>
@@ -5464,10 +5486,10 @@
     </row>
     <row r="337" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B337" s="8" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="C337" s="6" t="s">
         <v>119</v>
@@ -5475,10 +5497,10 @@
     </row>
     <row r="338" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B338" s="8" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="C338" s="6" t="s">
         <v>119</v>
@@ -5486,10 +5508,10 @@
     </row>
     <row r="339" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B339" s="8" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="C339" s="6" t="s">
         <v>119</v>
@@ -5497,10 +5519,10 @@
     </row>
     <row r="340" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B340" s="8" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="C340" s="6" t="s">
         <v>119</v>
@@ -5508,10 +5530,10 @@
     </row>
     <row r="341" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B341" s="8" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="C341" s="6" t="s">
         <v>119</v>
@@ -5519,10 +5541,10 @@
     </row>
     <row r="342" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B342" s="8" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="C342" s="6" t="s">
         <v>119</v>
@@ -5530,10 +5552,10 @@
     </row>
     <row r="343" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B343" s="8" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="C343" s="6" t="s">
         <v>119</v>
@@ -5541,10 +5563,10 @@
     </row>
     <row r="344" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B344" s="12" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="C344" s="6" t="s">
         <v>119</v>
@@ -5552,10 +5574,10 @@
     </row>
     <row r="345" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B345" s="8" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="C345" s="6" t="s">
         <v>119</v>
@@ -5563,10 +5585,10 @@
     </row>
     <row r="346" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A346" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B346" s="8" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="C346" s="6" t="s">
         <v>119</v>
@@ -5574,10 +5596,10 @@
     </row>
     <row r="347" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B347" s="8" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="C347" s="6" t="s">
         <v>119</v>
@@ -5585,10 +5607,10 @@
     </row>
     <row r="348" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A348" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B348" s="8" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="C348" s="6" t="s">
         <v>119</v>
@@ -5596,10 +5618,10 @@
     </row>
     <row r="349" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A349" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B349" s="8" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="C349" s="6" t="s">
         <v>119</v>
@@ -5607,10 +5629,10 @@
     </row>
     <row r="350" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A350" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B350" s="8" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="C350" s="6" t="s">
         <v>119</v>
@@ -5618,10 +5640,10 @@
     </row>
     <row r="351" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A351" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B351" s="8" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="C351" s="6" t="s">
         <v>119</v>
@@ -5629,10 +5651,10 @@
     </row>
     <row r="352" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A352" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B352" s="8" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="C352" s="6" t="s">
         <v>119</v>
@@ -5640,10 +5662,10 @@
     </row>
     <row r="353" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A353" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="B353" s="8" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="C353" s="6" t="s">
         <v>119</v>
@@ -5662,10 +5684,10 @@
     </row>
     <row r="356" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B356" s="8" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="C356" s="6" t="s">
         <v>119</v>
@@ -5673,10 +5695,10 @@
     </row>
     <row r="357" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B357" s="8" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="C357" s="6" t="s">
         <v>119</v>
@@ -5684,10 +5706,10 @@
     </row>
     <row r="358" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B358" s="8" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C358" s="6" t="s">
         <v>119</v>
@@ -5695,10 +5717,10 @@
     </row>
     <row r="359" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B359" s="8" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="C359" s="6" t="s">
         <v>119</v>
@@ -5706,10 +5728,10 @@
     </row>
     <row r="360" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A360" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B360" s="8" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="C360" s="6" t="s">
         <v>119</v>
@@ -5717,10 +5739,10 @@
     </row>
     <row r="361" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B361" s="8" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="C361" s="6" t="s">
         <v>119</v>
@@ -5728,10 +5750,10 @@
     </row>
     <row r="362" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A362" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B362" s="8" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="C362" s="6" t="s">
         <v>119</v>
@@ -5739,10 +5761,10 @@
     </row>
     <row r="363" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B363" s="8" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="C363" s="6" t="s">
         <v>119</v>
@@ -5750,10 +5772,10 @@
     </row>
     <row r="364" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B364" s="8" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="C364" s="6" t="s">
         <v>119</v>
@@ -5761,10 +5783,10 @@
     </row>
     <row r="365" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B365" s="8" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C365" s="6" t="s">
         <v>119</v>
@@ -5772,10 +5794,10 @@
     </row>
     <row r="366" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A366" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B366" s="8" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="C366" s="6" t="s">
         <v>119</v>
@@ -5783,10 +5805,10 @@
     </row>
     <row r="367" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B367" s="8" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="C367" s="6" t="s">
         <v>119</v>
@@ -5794,10 +5816,10 @@
     </row>
     <row r="368" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A368" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B368" s="8" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="C368" s="6" t="s">
         <v>119</v>
@@ -5805,10 +5827,10 @@
     </row>
     <row r="369" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A369" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B369" s="8" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="C369" s="6" t="s">
         <v>119</v>
@@ -5816,10 +5838,10 @@
     </row>
     <row r="370" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A370" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B370" s="8" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="C370" s="6" t="s">
         <v>119</v>
@@ -5827,10 +5849,10 @@
     </row>
     <row r="371" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B371" s="8" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="C371" s="6" t="s">
         <v>119</v>
@@ -5838,10 +5860,10 @@
     </row>
     <row r="372" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B372" s="8" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="C372" s="6" t="s">
         <v>119</v>
@@ -5849,10 +5871,10 @@
     </row>
     <row r="373" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B373" s="8" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="C373" s="6" t="s">
         <v>119</v>
@@ -5860,10 +5882,10 @@
     </row>
     <row r="374" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B374" s="8" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="C374" s="6" t="s">
         <v>119</v>
@@ -5871,10 +5893,10 @@
     </row>
     <row r="375" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B375" s="8" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="C375" s="6" t="s">
         <v>119</v>
@@ -5882,10 +5904,10 @@
     </row>
     <row r="376" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B376" s="8" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="C376" s="6" t="s">
         <v>119</v>
@@ -5893,10 +5915,10 @@
     </row>
     <row r="377" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B377" s="8" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="C377" s="6" t="s">
         <v>119</v>
@@ -5904,10 +5926,10 @@
     </row>
     <row r="378" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B378" s="8" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C378" s="6" t="s">
         <v>119</v>
@@ -5915,10 +5937,10 @@
     </row>
     <row r="379" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B379" s="8" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="C379" s="6" t="s">
         <v>119</v>
@@ -5926,10 +5948,10 @@
     </row>
     <row r="380" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A380" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B380" s="8" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="C380" s="6" t="s">
         <v>119</v>
@@ -5937,10 +5959,10 @@
     </row>
     <row r="381" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B381" s="8" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="C381" s="6" t="s">
         <v>119</v>
@@ -5948,10 +5970,10 @@
     </row>
     <row r="382" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B382" s="8" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="C382" s="6" t="s">
         <v>119</v>
@@ -5959,10 +5981,10 @@
     </row>
     <row r="383" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B383" s="8" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="C383" s="6" t="s">
         <v>119</v>
@@ -5970,10 +5992,10 @@
     </row>
     <row r="384" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B384" s="8" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="C384" s="6" t="s">
         <v>119</v>
@@ -5981,10 +6003,10 @@
     </row>
     <row r="385" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B385" s="8" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="C385" s="6" t="s">
         <v>119</v>
@@ -5992,10 +6014,10 @@
     </row>
     <row r="386" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B386" s="8" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="C386" s="6" t="s">
         <v>119</v>
@@ -6003,10 +6025,10 @@
     </row>
     <row r="387" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B387" s="8" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="C387" s="6" t="s">
         <v>119</v>
@@ -6014,10 +6036,10 @@
     </row>
     <row r="388" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B388" s="8" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="C388" s="6" t="s">
         <v>119</v>
@@ -6025,10 +6047,10 @@
     </row>
     <row r="389" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B389" s="8" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="C389" s="6" t="s">
         <v>119</v>
@@ -6036,10 +6058,10 @@
     </row>
     <row r="390" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B390" s="8" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="C390" s="6" t="s">
         <v>119</v>
@@ -6047,10 +6069,10 @@
     </row>
     <row r="391" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B391" s="8" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="C391" s="6" t="s">
         <v>119</v>
@@ -6058,10 +6080,10 @@
     </row>
     <row r="392" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B392" s="8" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="C392" s="6" t="s">
         <v>119</v>
@@ -6069,10 +6091,10 @@
     </row>
     <row r="393" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B393" s="8" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="C393" s="6" t="s">
         <v>119</v>
@@ -6080,10 +6102,10 @@
     </row>
     <row r="394" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B394" s="8" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="C394" s="6" t="s">
         <v>119</v>
@@ -6091,10 +6113,10 @@
     </row>
     <row r="395" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B395" s="8" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="C395" s="6" t="s">
         <v>119</v>
@@ -6102,10 +6124,10 @@
     </row>
     <row r="396" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B396" s="8" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="C396" s="6" t="s">
         <v>119</v>
@@ -6113,10 +6135,10 @@
     </row>
     <row r="397" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B397" s="8" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="C397" s="6" t="s">
         <v>119</v>
@@ -6124,10 +6146,10 @@
     </row>
     <row r="398" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B398" s="8" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="C398" s="6" t="s">
         <v>119</v>
@@ -6135,10 +6157,10 @@
     </row>
     <row r="399" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="7" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="B399" s="8" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="C399" s="6" t="s">
         <v>119</v>
@@ -6157,10 +6179,10 @@
     </row>
     <row r="402" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B402" s="8" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C402" s="6" t="s">
         <v>119</v>
@@ -6168,10 +6190,10 @@
     </row>
     <row r="403" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B403" s="8" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="C403" s="6" t="s">
         <v>119</v>
@@ -6179,10 +6201,10 @@
     </row>
     <row r="404" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B404" s="8" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="C404" s="6" t="s">
         <v>119</v>
@@ -6190,7 +6212,7 @@
     </row>
     <row r="405" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A405" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B405" s="8" t="s">
         <v>122</v>
@@ -6201,10 +6223,10 @@
     </row>
     <row r="406" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B406" s="8" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="C406" s="6" t="s">
         <v>119</v>
@@ -6212,10 +6234,10 @@
     </row>
     <row r="407" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A407" s="7" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="B407" s="8" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="C407" s="6" t="s">
         <v>119</v>
@@ -6234,10 +6256,10 @@
     </row>
     <row r="410" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B410" s="8" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="C410" s="6" t="s">
         <v>119</v>
@@ -6245,10 +6267,10 @@
     </row>
     <row r="411" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B411" s="8" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="C411" s="6" t="s">
         <v>119</v>
@@ -6256,10 +6278,10 @@
     </row>
     <row r="412" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B412" s="8" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="C412" s="6" t="s">
         <v>119</v>
@@ -6267,10 +6289,10 @@
     </row>
     <row r="413" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="C413" s="6" t="s">
         <v>119</v>
@@ -6278,10 +6300,10 @@
     </row>
     <row r="414" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="C414" s="6" t="s">
         <v>119</v>
@@ -6289,10 +6311,10 @@
     </row>
     <row r="415" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B415" s="8" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C415" s="6" t="s">
         <v>119</v>
@@ -6300,10 +6322,10 @@
     </row>
     <row r="416" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B416" s="8" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="C416" s="6" t="s">
         <v>119</v>
@@ -6311,10 +6333,10 @@
     </row>
     <row r="417" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B417" s="8" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="C417" s="6" t="s">
         <v>119</v>
@@ -6322,10 +6344,10 @@
     </row>
     <row r="418" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B418" s="8" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="C418" s="6" t="s">
         <v>119</v>
@@ -6333,10 +6355,10 @@
     </row>
     <row r="419" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="C419" s="6" t="s">
         <v>119</v>
@@ -6344,10 +6366,10 @@
     </row>
     <row r="420" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B420" s="8" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="C420" s="6" t="s">
         <v>119</v>
@@ -6355,10 +6377,10 @@
     </row>
     <row r="421" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B421" s="8" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="C421" s="6" t="s">
         <v>119</v>
@@ -6366,10 +6388,10 @@
     </row>
     <row r="422" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="C422" s="6" t="s">
         <v>119</v>
@@ -6377,10 +6399,10 @@
     </row>
     <row r="423" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B423" s="8" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="C423" s="6" t="s">
         <v>119</v>
@@ -6388,10 +6410,10 @@
     </row>
     <row r="424" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B424" s="8" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="C424" s="6" t="s">
         <v>119</v>
@@ -6399,10 +6421,10 @@
     </row>
     <row r="425" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B425" s="8" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="C425" s="6" t="s">
         <v>119</v>
@@ -6410,10 +6432,10 @@
     </row>
     <row r="426" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B426" s="8" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="C426" s="6" t="s">
         <v>119</v>
@@ -6421,10 +6443,10 @@
     </row>
     <row r="427" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B427" s="8" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="C427" s="6" t="s">
         <v>119</v>
@@ -6432,10 +6454,10 @@
     </row>
     <row r="428" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B428" s="8" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="C428" s="6" t="s">
         <v>119</v>
@@ -6443,10 +6465,10 @@
     </row>
     <row r="429" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B429" s="8" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="C429" s="6" t="s">
         <v>119</v>
@@ -6454,10 +6476,10 @@
     </row>
     <row r="430" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B430" s="8" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="C430" s="6" t="s">
         <v>119</v>
@@ -6465,10 +6487,10 @@
     </row>
     <row r="431" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B431" s="8" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="C431" s="6" t="s">
         <v>119</v>
@@ -6476,10 +6498,10 @@
     </row>
     <row r="432" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B432" s="8" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="C432" s="6" t="s">
         <v>119</v>
@@ -6487,10 +6509,10 @@
     </row>
     <row r="433" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B433" s="8" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="C433" s="6" t="s">
         <v>119</v>
@@ -6498,10 +6520,10 @@
     </row>
     <row r="434" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B434" s="8" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="C434" s="6" t="s">
         <v>119</v>
@@ -6509,10 +6531,10 @@
     </row>
     <row r="435" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A435" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B435" s="8" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="C435" s="6" t="s">
         <v>119</v>
@@ -6520,10 +6542,10 @@
     </row>
     <row r="436" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B436" s="8" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="C436" s="6" t="s">
         <v>119</v>
@@ -6531,10 +6553,10 @@
     </row>
     <row r="437" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B437" s="8" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="C437" s="6" t="s">
         <v>119</v>
@@ -6542,10 +6564,10 @@
     </row>
     <row r="438" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B438" s="8" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C438" s="6" t="s">
         <v>119</v>
@@ -6553,10 +6575,10 @@
     </row>
     <row r="439" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B439" s="8" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="C439" s="6" t="s">
         <v>119</v>
@@ -6564,10 +6586,10 @@
     </row>
     <row r="440" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B440" s="8" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="C440" s="6" t="s">
         <v>119</v>
@@ -6575,10 +6597,10 @@
     </row>
     <row r="441" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B441" s="8" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="C441" s="6" t="s">
         <v>119</v>
@@ -6586,10 +6608,10 @@
     </row>
     <row r="442" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B442" s="8" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="C442" s="6" t="s">
         <v>119</v>
@@ -6597,10 +6619,10 @@
     </row>
     <row r="443" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B443" s="8" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="C443" s="6" t="s">
         <v>119</v>
@@ -6608,10 +6630,10 @@
     </row>
     <row r="444" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B444" s="8" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="C444" s="6" t="s">
         <v>119</v>
@@ -6619,10 +6641,10 @@
     </row>
     <row r="445" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B445" s="8" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="C445" s="6" t="s">
         <v>119</v>
@@ -6630,10 +6652,10 @@
     </row>
     <row r="446" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B446" s="8" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="C446" s="6" t="s">
         <v>119</v>
@@ -6641,10 +6663,10 @@
     </row>
     <row r="447" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B447" s="8" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="C447" s="6" t="s">
         <v>119</v>
@@ -6652,10 +6674,10 @@
     </row>
     <row r="448" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B448" s="8" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="C448" s="6" t="s">
         <v>119</v>
@@ -6663,10 +6685,10 @@
     </row>
     <row r="449" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B449" s="8" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="C449" s="6" t="s">
         <v>119</v>
@@ -6674,10 +6696,10 @@
     </row>
     <row r="450" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B450" s="8" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="C450" s="6" t="s">
         <v>119</v>
@@ -6685,10 +6707,10 @@
     </row>
     <row r="451" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B451" s="8" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
       <c r="C451" s="6" t="s">
         <v>119</v>
@@ -6696,10 +6718,10 @@
     </row>
     <row r="452" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B452" s="8" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="C452" s="6" t="s">
         <v>119</v>
@@ -6707,10 +6729,10 @@
     </row>
     <row r="453" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A453" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B453" s="8" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
       <c r="C453" s="6" t="s">
         <v>119</v>
@@ -6718,10 +6740,10 @@
     </row>
     <row r="454" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B454" s="8" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="C454" s="6" t="s">
         <v>119</v>
@@ -6729,10 +6751,10 @@
     </row>
     <row r="455" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B455" s="8" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="C455" s="6" t="s">
         <v>119</v>
@@ -6740,10 +6762,10 @@
     </row>
     <row r="456" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B456" s="8" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="C456" s="6" t="s">
         <v>119</v>
@@ -6751,10 +6773,10 @@
     </row>
     <row r="457" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B457" s="8" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
       <c r="C457" s="6" t="s">
         <v>119</v>
@@ -6762,10 +6784,10 @@
     </row>
     <row r="458" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B458" s="8" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
       <c r="C458" s="6" t="s">
         <v>119</v>
@@ -6773,10 +6795,10 @@
     </row>
     <row r="459" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A459" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B459" s="8" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="C459" s="6" t="s">
         <v>119</v>
@@ -6784,10 +6806,10 @@
     </row>
     <row r="460" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B460" s="8" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="C460" s="6" t="s">
         <v>119</v>
@@ -6795,10 +6817,10 @@
     </row>
     <row r="461" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B461" s="8" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="C461" s="6" t="s">
         <v>119</v>
@@ -6806,10 +6828,10 @@
     </row>
     <row r="462" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B462" s="8" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="C462" s="6" t="s">
         <v>119</v>
@@ -6817,10 +6839,10 @@
     </row>
     <row r="463" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B463" s="8" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
       <c r="C463" s="6" t="s">
         <v>119</v>
@@ -6828,10 +6850,10 @@
     </row>
     <row r="464" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B464" s="8" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="C464" s="6" t="s">
         <v>119</v>
@@ -6839,10 +6861,10 @@
     </row>
     <row r="465" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B465" s="8" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="C465" s="6" t="s">
         <v>119</v>
@@ -6850,10 +6872,10 @@
     </row>
     <row r="466" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B466" s="8" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="C466" s="6" t="s">
         <v>119</v>
@@ -6861,10 +6883,10 @@
     </row>
     <row r="467" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B467" s="8" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="C467" s="6" t="s">
         <v>119</v>
@@ -6872,10 +6894,10 @@
     </row>
     <row r="468" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B468" s="8" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="C468" s="6" t="s">
         <v>119</v>
@@ -6883,10 +6905,10 @@
     </row>
     <row r="469" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="7" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="B469" s="8" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="C469" s="6" t="s">
         <v>119</v>
@@ -6905,10 +6927,10 @@
     </row>
     <row r="472" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B472" s="8" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="C472" s="6" t="s">
         <v>119</v>
@@ -6916,10 +6938,10 @@
     </row>
     <row r="473" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B473" s="8" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="C473" s="6" t="s">
         <v>119</v>
@@ -6927,10 +6949,10 @@
     </row>
     <row r="474" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B474" s="8" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
       <c r="C474" s="6" t="s">
         <v>119</v>
@@ -6938,10 +6960,10 @@
     </row>
     <row r="475" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B475" s="8" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="C475" s="6" t="s">
         <v>119</v>
@@ -6949,10 +6971,10 @@
     </row>
     <row r="476" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B476" s="8" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="C476" s="6" t="s">
         <v>119</v>
@@ -6960,10 +6982,10 @@
     </row>
     <row r="477" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B477" s="8" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="C477" s="6" t="s">
         <v>119</v>
@@ -6971,10 +6993,10 @@
     </row>
     <row r="478" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B478" s="8" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="C478" s="6" t="s">
         <v>119</v>
@@ -6982,10 +7004,10 @@
     </row>
     <row r="479" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B479" s="8" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
       <c r="C479" s="6" t="s">
         <v>119</v>
@@ -6993,10 +7015,10 @@
     </row>
     <row r="480" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B480" s="8" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="C480" s="6" t="s">
         <v>119</v>
@@ -7004,10 +7026,10 @@
     </row>
     <row r="481" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="7" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B481" s="8" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="C481" s="6" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
Heap completed and minor change in Linked List problem
</commit_message>
<xml_diff>
--- a/FINAL450.xlsx
+++ b/FINAL450.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="532">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="541">
   <si>
     <t xml:space="preserve">YES(Iterative &amp; recursive)</t>
   </si>
@@ -1237,18 +1237,30 @@
     <t xml:space="preserve">Sort an Array using heap. (HeapSort)</t>
   </si>
   <si>
+    <t xml:space="preserve">y(as above with repeatation)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum of all subarrays of size k.</t>
   </si>
   <si>
     <t xml:space="preserve">“k” largest element in an array</t>
   </si>
   <si>
+    <t xml:space="preserve">y(this and next similar)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kth smallest and largest element in an unsorted array</t>
   </si>
   <si>
+    <t xml:space="preserve">y(this and previous similar)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Merge “K” sorted arrays. [ IMP ]</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(1st kElmntsFrmEachRplc 1  rmvdFrmSmArray)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Merge 2 Binary Max Heaps</t>
   </si>
   <si>
@@ -1261,12 +1273,21 @@
     <t xml:space="preserve">Merge “K” Sorted Linked Lists [V.IMP]</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Using priority queue)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Smallest range in “K” Lists</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(traverse&amp;pushMinheap,untilAtlst1ArrayEnds)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Median in a stream of Integers</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(both balanced min max heap)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Check if a Binary Tree is Heap</t>
   </si>
   <si>
@@ -1276,10 +1297,16 @@
     <t xml:space="preserve">Convert BST to Min Heap</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(inorder then preorder)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Convert min heap to max heap</t>
   </si>
   <si>
     <t xml:space="preserve">Rearrange characters in a string such that no two adjacent are same.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">y(done leetcode reorganize string)</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum sum of two numbers formed from digits of an array</t>
@@ -1928,7 +1955,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C481"/>
-  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="111.76"/>
@@ -4197,7 +4224,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="7" t="s">
         <v>268</v>
       </c>
@@ -4274,7 +4301,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A223" s="7" t="s">
         <v>268</v>
       </c>
@@ -4296,7 +4323,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="7" t="s">
         <v>268</v>
       </c>
@@ -4329,7 +4356,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="7" t="s">
         <v>268</v>
       </c>
@@ -4362,7 +4389,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="7" t="s">
         <v>268</v>
       </c>
@@ -4395,7 +4422,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="7" t="s">
         <v>268</v>
       </c>
@@ -4406,7 +4433,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="7" t="s">
         <v>268</v>
       </c>
@@ -5481,7 +5508,7 @@
         <v>393</v>
       </c>
       <c r="C336" s="6" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="337" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5492,7 +5519,7 @@
         <v>394</v>
       </c>
       <c r="C337" s="6" t="s">
-        <v>119</v>
+        <v>395</v>
       </c>
     </row>
     <row r="338" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5500,10 +5527,10 @@
         <v>392</v>
       </c>
       <c r="B338" s="8" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C338" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="339" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5511,10 +5538,10 @@
         <v>392</v>
       </c>
       <c r="B339" s="8" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C339" s="6" t="s">
-        <v>119</v>
+        <v>398</v>
       </c>
     </row>
     <row r="340" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5522,10 +5549,10 @@
         <v>392</v>
       </c>
       <c r="B340" s="8" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="C340" s="6" t="s">
-        <v>119</v>
+        <v>400</v>
       </c>
     </row>
     <row r="341" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5533,10 +5560,10 @@
         <v>392</v>
       </c>
       <c r="B341" s="8" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="C341" s="6" t="s">
-        <v>119</v>
+        <v>402</v>
       </c>
     </row>
     <row r="342" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5544,10 +5571,10 @@
         <v>392</v>
       </c>
       <c r="B342" s="8" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="C342" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="343" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5555,10 +5582,10 @@
         <v>392</v>
       </c>
       <c r="B343" s="8" t="s">
-        <v>400</v>
-      </c>
-      <c r="C343" s="6" t="s">
-        <v>119</v>
+        <v>404</v>
+      </c>
+      <c r="C343" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="344" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5566,10 +5593,10 @@
         <v>392</v>
       </c>
       <c r="B344" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="C344" s="6" t="s">
-        <v>119</v>
+        <v>405</v>
+      </c>
+      <c r="C344" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="345" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5577,10 +5604,10 @@
         <v>392</v>
       </c>
       <c r="B345" s="8" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="C345" s="6" t="s">
-        <v>119</v>
+        <v>407</v>
       </c>
     </row>
     <row r="346" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5588,21 +5615,21 @@
         <v>392</v>
       </c>
       <c r="B346" s="8" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="C346" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="347" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="347" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="7" t="s">
         <v>392</v>
       </c>
       <c r="B347" s="8" t="s">
-        <v>404</v>
-      </c>
-      <c r="C347" s="6" t="s">
-        <v>119</v>
+        <v>410</v>
+      </c>
+      <c r="C347" s="9" t="s">
+        <v>411</v>
       </c>
     </row>
     <row r="348" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5610,10 +5637,10 @@
         <v>392</v>
       </c>
       <c r="B348" s="8" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="C348" s="6" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="349" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5621,10 +5648,10 @@
         <v>392</v>
       </c>
       <c r="B349" s="8" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="C349" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="350" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5632,10 +5659,10 @@
         <v>392</v>
       </c>
       <c r="B350" s="8" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="C350" s="6" t="s">
-        <v>119</v>
+        <v>415</v>
       </c>
     </row>
     <row r="351" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5643,10 +5670,10 @@
         <v>392</v>
       </c>
       <c r="B351" s="8" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="C351" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="352" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5654,10 +5681,10 @@
         <v>392</v>
       </c>
       <c r="B352" s="8" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C352" s="6" t="s">
-        <v>119</v>
+        <v>418</v>
       </c>
     </row>
     <row r="353" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5665,10 +5692,10 @@
         <v>392</v>
       </c>
       <c r="B353" s="8" t="s">
-        <v>410</v>
+        <v>419</v>
       </c>
       <c r="C353" s="6" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="354" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5684,10 +5711,10 @@
     </row>
     <row r="356" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A356" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B356" s="8" t="s">
-        <v>412</v>
+        <v>421</v>
       </c>
       <c r="C356" s="6" t="s">
         <v>119</v>
@@ -5695,10 +5722,10 @@
     </row>
     <row r="357" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A357" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B357" s="8" t="s">
-        <v>413</v>
+        <v>422</v>
       </c>
       <c r="C357" s="6" t="s">
         <v>119</v>
@@ -5706,10 +5733,10 @@
     </row>
     <row r="358" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B358" s="8" t="s">
-        <v>414</v>
+        <v>423</v>
       </c>
       <c r="C358" s="6" t="s">
         <v>119</v>
@@ -5717,10 +5744,10 @@
     </row>
     <row r="359" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B359" s="8" t="s">
-        <v>415</v>
+        <v>424</v>
       </c>
       <c r="C359" s="6" t="s">
         <v>119</v>
@@ -5728,10 +5755,10 @@
     </row>
     <row r="360" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A360" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B360" s="8" t="s">
-        <v>416</v>
+        <v>425</v>
       </c>
       <c r="C360" s="6" t="s">
         <v>119</v>
@@ -5739,10 +5766,10 @@
     </row>
     <row r="361" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B361" s="8" t="s">
-        <v>417</v>
+        <v>426</v>
       </c>
       <c r="C361" s="6" t="s">
         <v>119</v>
@@ -5750,10 +5777,10 @@
     </row>
     <row r="362" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A362" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B362" s="8" t="s">
-        <v>418</v>
+        <v>427</v>
       </c>
       <c r="C362" s="6" t="s">
         <v>119</v>
@@ -5761,10 +5788,10 @@
     </row>
     <row r="363" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B363" s="8" t="s">
-        <v>419</v>
+        <v>428</v>
       </c>
       <c r="C363" s="6" t="s">
         <v>119</v>
@@ -5772,10 +5799,10 @@
     </row>
     <row r="364" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B364" s="8" t="s">
-        <v>420</v>
+        <v>429</v>
       </c>
       <c r="C364" s="6" t="s">
         <v>119</v>
@@ -5783,10 +5810,10 @@
     </row>
     <row r="365" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B365" s="8" t="s">
-        <v>421</v>
+        <v>430</v>
       </c>
       <c r="C365" s="6" t="s">
         <v>119</v>
@@ -5794,10 +5821,10 @@
     </row>
     <row r="366" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A366" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B366" s="8" t="s">
-        <v>422</v>
+        <v>431</v>
       </c>
       <c r="C366" s="6" t="s">
         <v>119</v>
@@ -5805,10 +5832,10 @@
     </row>
     <row r="367" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B367" s="8" t="s">
-        <v>423</v>
+        <v>432</v>
       </c>
       <c r="C367" s="6" t="s">
         <v>119</v>
@@ -5816,10 +5843,10 @@
     </row>
     <row r="368" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A368" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B368" s="8" t="s">
-        <v>424</v>
+        <v>433</v>
       </c>
       <c r="C368" s="6" t="s">
         <v>119</v>
@@ -5827,10 +5854,10 @@
     </row>
     <row r="369" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A369" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B369" s="8" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="C369" s="6" t="s">
         <v>119</v>
@@ -5838,10 +5865,10 @@
     </row>
     <row r="370" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A370" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B370" s="8" t="s">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="C370" s="6" t="s">
         <v>119</v>
@@ -5849,10 +5876,10 @@
     </row>
     <row r="371" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B371" s="8" t="s">
-        <v>427</v>
+        <v>436</v>
       </c>
       <c r="C371" s="6" t="s">
         <v>119</v>
@@ -5860,10 +5887,10 @@
     </row>
     <row r="372" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B372" s="8" t="s">
-        <v>428</v>
+        <v>437</v>
       </c>
       <c r="C372" s="6" t="s">
         <v>119</v>
@@ -5871,10 +5898,10 @@
     </row>
     <row r="373" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B373" s="8" t="s">
-        <v>429</v>
+        <v>438</v>
       </c>
       <c r="C373" s="6" t="s">
         <v>119</v>
@@ -5882,10 +5909,10 @@
     </row>
     <row r="374" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B374" s="8" t="s">
-        <v>430</v>
+        <v>439</v>
       </c>
       <c r="C374" s="6" t="s">
         <v>119</v>
@@ -5893,10 +5920,10 @@
     </row>
     <row r="375" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B375" s="8" t="s">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="C375" s="6" t="s">
         <v>119</v>
@@ -5904,10 +5931,10 @@
     </row>
     <row r="376" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B376" s="8" t="s">
-        <v>432</v>
+        <v>441</v>
       </c>
       <c r="C376" s="6" t="s">
         <v>119</v>
@@ -5915,10 +5942,10 @@
     </row>
     <row r="377" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B377" s="8" t="s">
-        <v>433</v>
+        <v>442</v>
       </c>
       <c r="C377" s="6" t="s">
         <v>119</v>
@@ -5926,10 +5953,10 @@
     </row>
     <row r="378" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B378" s="8" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="C378" s="6" t="s">
         <v>119</v>
@@ -5937,10 +5964,10 @@
     </row>
     <row r="379" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B379" s="8" t="s">
-        <v>435</v>
+        <v>444</v>
       </c>
       <c r="C379" s="6" t="s">
         <v>119</v>
@@ -5948,10 +5975,10 @@
     </row>
     <row r="380" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A380" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B380" s="8" t="s">
-        <v>436</v>
+        <v>445</v>
       </c>
       <c r="C380" s="6" t="s">
         <v>119</v>
@@ -5959,10 +5986,10 @@
     </row>
     <row r="381" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B381" s="8" t="s">
-        <v>437</v>
+        <v>446</v>
       </c>
       <c r="C381" s="6" t="s">
         <v>119</v>
@@ -5970,10 +5997,10 @@
     </row>
     <row r="382" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B382" s="8" t="s">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="C382" s="6" t="s">
         <v>119</v>
@@ -5981,10 +6008,10 @@
     </row>
     <row r="383" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B383" s="8" t="s">
-        <v>439</v>
+        <v>448</v>
       </c>
       <c r="C383" s="6" t="s">
         <v>119</v>
@@ -5992,10 +6019,10 @@
     </row>
     <row r="384" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B384" s="8" t="s">
-        <v>440</v>
+        <v>449</v>
       </c>
       <c r="C384" s="6" t="s">
         <v>119</v>
@@ -6003,10 +6030,10 @@
     </row>
     <row r="385" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B385" s="8" t="s">
-        <v>441</v>
+        <v>450</v>
       </c>
       <c r="C385" s="6" t="s">
         <v>119</v>
@@ -6014,10 +6041,10 @@
     </row>
     <row r="386" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B386" s="8" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="C386" s="6" t="s">
         <v>119</v>
@@ -6025,10 +6052,10 @@
     </row>
     <row r="387" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B387" s="8" t="s">
-        <v>443</v>
+        <v>452</v>
       </c>
       <c r="C387" s="6" t="s">
         <v>119</v>
@@ -6036,10 +6063,10 @@
     </row>
     <row r="388" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B388" s="8" t="s">
-        <v>444</v>
+        <v>453</v>
       </c>
       <c r="C388" s="6" t="s">
         <v>119</v>
@@ -6047,10 +6074,10 @@
     </row>
     <row r="389" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B389" s="8" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
       <c r="C389" s="6" t="s">
         <v>119</v>
@@ -6058,10 +6085,10 @@
     </row>
     <row r="390" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B390" s="8" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
       <c r="C390" s="6" t="s">
         <v>119</v>
@@ -6069,10 +6096,10 @@
     </row>
     <row r="391" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B391" s="8" t="s">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="C391" s="6" t="s">
         <v>119</v>
@@ -6080,10 +6107,10 @@
     </row>
     <row r="392" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B392" s="8" t="s">
-        <v>447</v>
+        <v>456</v>
       </c>
       <c r="C392" s="6" t="s">
         <v>119</v>
@@ -6091,10 +6118,10 @@
     </row>
     <row r="393" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B393" s="8" t="s">
-        <v>448</v>
+        <v>457</v>
       </c>
       <c r="C393" s="6" t="s">
         <v>119</v>
@@ -6102,10 +6129,10 @@
     </row>
     <row r="394" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B394" s="8" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="C394" s="6" t="s">
         <v>119</v>
@@ -6113,10 +6140,10 @@
     </row>
     <row r="395" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B395" s="8" t="s">
-        <v>450</v>
+        <v>459</v>
       </c>
       <c r="C395" s="6" t="s">
         <v>119</v>
@@ -6124,10 +6151,10 @@
     </row>
     <row r="396" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B396" s="8" t="s">
-        <v>451</v>
+        <v>460</v>
       </c>
       <c r="C396" s="6" t="s">
         <v>119</v>
@@ -6135,10 +6162,10 @@
     </row>
     <row r="397" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B397" s="8" t="s">
-        <v>452</v>
+        <v>461</v>
       </c>
       <c r="C397" s="6" t="s">
         <v>119</v>
@@ -6146,10 +6173,10 @@
     </row>
     <row r="398" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B398" s="8" t="s">
-        <v>453</v>
+        <v>462</v>
       </c>
       <c r="C398" s="6" t="s">
         <v>119</v>
@@ -6157,10 +6184,10 @@
     </row>
     <row r="399" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="7" t="s">
-        <v>411</v>
+        <v>420</v>
       </c>
       <c r="B399" s="8" t="s">
-        <v>454</v>
+        <v>463</v>
       </c>
       <c r="C399" s="6" t="s">
         <v>119</v>
@@ -6179,10 +6206,10 @@
     </row>
     <row r="402" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="7" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="B402" s="8" t="s">
-        <v>456</v>
+        <v>465</v>
       </c>
       <c r="C402" s="6" t="s">
         <v>119</v>
@@ -6190,10 +6217,10 @@
     </row>
     <row r="403" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="7" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="B403" s="8" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="C403" s="6" t="s">
         <v>119</v>
@@ -6201,10 +6228,10 @@
     </row>
     <row r="404" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="7" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="B404" s="8" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="C404" s="6" t="s">
         <v>119</v>
@@ -6212,7 +6239,7 @@
     </row>
     <row r="405" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A405" s="7" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="B405" s="8" t="s">
         <v>122</v>
@@ -6223,10 +6250,10 @@
     </row>
     <row r="406" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="7" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="B406" s="8" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="C406" s="6" t="s">
         <v>119</v>
@@ -6234,10 +6261,10 @@
     </row>
     <row r="407" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A407" s="7" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
       <c r="B407" s="8" t="s">
-        <v>460</v>
+        <v>469</v>
       </c>
       <c r="C407" s="6" t="s">
         <v>119</v>
@@ -6256,10 +6283,10 @@
     </row>
     <row r="410" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B410" s="8" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
       <c r="C410" s="6" t="s">
         <v>119</v>
@@ -6267,10 +6294,10 @@
     </row>
     <row r="411" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B411" s="8" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
       <c r="C411" s="6" t="s">
         <v>119</v>
@@ -6278,10 +6305,10 @@
     </row>
     <row r="412" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B412" s="8" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
       <c r="C412" s="6" t="s">
         <v>119</v>
@@ -6289,10 +6316,10 @@
     </row>
     <row r="413" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="C413" s="6" t="s">
         <v>119</v>
@@ -6300,10 +6327,10 @@
     </row>
     <row r="414" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="C414" s="6" t="s">
         <v>119</v>
@@ -6311,10 +6338,10 @@
     </row>
     <row r="415" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B415" s="8" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
       <c r="C415" s="6" t="s">
         <v>119</v>
@@ -6322,10 +6349,10 @@
     </row>
     <row r="416" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B416" s="8" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="C416" s="6" t="s">
         <v>119</v>
@@ -6333,7 +6360,7 @@
     </row>
     <row r="417" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B417" s="8" t="s">
         <v>341</v>
@@ -6344,10 +6371,10 @@
     </row>
     <row r="418" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B418" s="8" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="C418" s="6" t="s">
         <v>119</v>
@@ -6355,10 +6382,10 @@
     </row>
     <row r="419" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>470</v>
+        <v>479</v>
       </c>
       <c r="C419" s="6" t="s">
         <v>119</v>
@@ -6366,10 +6393,10 @@
     </row>
     <row r="420" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B420" s="8" t="s">
-        <v>471</v>
+        <v>480</v>
       </c>
       <c r="C420" s="6" t="s">
         <v>119</v>
@@ -6377,10 +6404,10 @@
     </row>
     <row r="421" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B421" s="8" t="s">
-        <v>472</v>
+        <v>481</v>
       </c>
       <c r="C421" s="6" t="s">
         <v>119</v>
@@ -6388,10 +6415,10 @@
     </row>
     <row r="422" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
       <c r="C422" s="6" t="s">
         <v>119</v>
@@ -6399,10 +6426,10 @@
     </row>
     <row r="423" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B423" s="8" t="s">
-        <v>474</v>
+        <v>483</v>
       </c>
       <c r="C423" s="6" t="s">
         <v>119</v>
@@ -6410,10 +6437,10 @@
     </row>
     <row r="424" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B424" s="8" t="s">
-        <v>475</v>
+        <v>484</v>
       </c>
       <c r="C424" s="6" t="s">
         <v>119</v>
@@ -6421,10 +6448,10 @@
     </row>
     <row r="425" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B425" s="8" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="C425" s="6" t="s">
         <v>119</v>
@@ -6432,10 +6459,10 @@
     </row>
     <row r="426" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B426" s="8" t="s">
-        <v>477</v>
+        <v>486</v>
       </c>
       <c r="C426" s="6" t="s">
         <v>119</v>
@@ -6443,10 +6470,10 @@
     </row>
     <row r="427" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B427" s="8" t="s">
-        <v>478</v>
+        <v>487</v>
       </c>
       <c r="C427" s="6" t="s">
         <v>119</v>
@@ -6454,10 +6481,10 @@
     </row>
     <row r="428" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B428" s="8" t="s">
-        <v>479</v>
+        <v>488</v>
       </c>
       <c r="C428" s="6" t="s">
         <v>119</v>
@@ -6465,10 +6492,10 @@
     </row>
     <row r="429" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B429" s="8" t="s">
-        <v>480</v>
+        <v>489</v>
       </c>
       <c r="C429" s="6" t="s">
         <v>119</v>
@@ -6476,10 +6503,10 @@
     </row>
     <row r="430" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B430" s="8" t="s">
-        <v>481</v>
+        <v>490</v>
       </c>
       <c r="C430" s="6" t="s">
         <v>119</v>
@@ -6487,10 +6514,10 @@
     </row>
     <row r="431" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B431" s="8" t="s">
-        <v>482</v>
+        <v>491</v>
       </c>
       <c r="C431" s="6" t="s">
         <v>119</v>
@@ -6498,10 +6525,10 @@
     </row>
     <row r="432" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B432" s="8" t="s">
-        <v>483</v>
+        <v>492</v>
       </c>
       <c r="C432" s="6" t="s">
         <v>119</v>
@@ -6509,10 +6536,10 @@
     </row>
     <row r="433" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B433" s="8" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="C433" s="6" t="s">
         <v>119</v>
@@ -6520,10 +6547,10 @@
     </row>
     <row r="434" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B434" s="8" t="s">
-        <v>485</v>
+        <v>494</v>
       </c>
       <c r="C434" s="6" t="s">
         <v>119</v>
@@ -6531,10 +6558,10 @@
     </row>
     <row r="435" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A435" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B435" s="8" t="s">
-        <v>486</v>
+        <v>495</v>
       </c>
       <c r="C435" s="6" t="s">
         <v>119</v>
@@ -6542,10 +6569,10 @@
     </row>
     <row r="436" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B436" s="8" t="s">
-        <v>487</v>
+        <v>496</v>
       </c>
       <c r="C436" s="6" t="s">
         <v>119</v>
@@ -6553,10 +6580,10 @@
     </row>
     <row r="437" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B437" s="8" t="s">
-        <v>488</v>
+        <v>497</v>
       </c>
       <c r="C437" s="6" t="s">
         <v>119</v>
@@ -6564,10 +6591,10 @@
     </row>
     <row r="438" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B438" s="8" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C438" s="6" t="s">
         <v>119</v>
@@ -6575,10 +6602,10 @@
     </row>
     <row r="439" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B439" s="8" t="s">
-        <v>490</v>
+        <v>499</v>
       </c>
       <c r="C439" s="6" t="s">
         <v>119</v>
@@ -6586,10 +6613,10 @@
     </row>
     <row r="440" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B440" s="8" t="s">
-        <v>491</v>
+        <v>500</v>
       </c>
       <c r="C440" s="6" t="s">
         <v>119</v>
@@ -6597,10 +6624,10 @@
     </row>
     <row r="441" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B441" s="8" t="s">
-        <v>492</v>
+        <v>501</v>
       </c>
       <c r="C441" s="6" t="s">
         <v>119</v>
@@ -6608,10 +6635,10 @@
     </row>
     <row r="442" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B442" s="8" t="s">
-        <v>493</v>
+        <v>502</v>
       </c>
       <c r="C442" s="6" t="s">
         <v>119</v>
@@ -6619,10 +6646,10 @@
     </row>
     <row r="443" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B443" s="8" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="C443" s="6" t="s">
         <v>119</v>
@@ -6630,10 +6657,10 @@
     </row>
     <row r="444" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B444" s="8" t="s">
-        <v>495</v>
+        <v>504</v>
       </c>
       <c r="C444" s="6" t="s">
         <v>119</v>
@@ -6641,10 +6668,10 @@
     </row>
     <row r="445" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B445" s="8" t="s">
-        <v>496</v>
+        <v>505</v>
       </c>
       <c r="C445" s="6" t="s">
         <v>119</v>
@@ -6652,10 +6679,10 @@
     </row>
     <row r="446" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B446" s="8" t="s">
-        <v>497</v>
+        <v>506</v>
       </c>
       <c r="C446" s="6" t="s">
         <v>119</v>
@@ -6663,10 +6690,10 @@
     </row>
     <row r="447" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B447" s="8" t="s">
-        <v>498</v>
+        <v>507</v>
       </c>
       <c r="C447" s="6" t="s">
         <v>119</v>
@@ -6674,10 +6701,10 @@
     </row>
     <row r="448" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B448" s="8" t="s">
-        <v>499</v>
+        <v>508</v>
       </c>
       <c r="C448" s="6" t="s">
         <v>119</v>
@@ -6685,10 +6712,10 @@
     </row>
     <row r="449" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B449" s="8" t="s">
-        <v>500</v>
+        <v>509</v>
       </c>
       <c r="C449" s="6" t="s">
         <v>119</v>
@@ -6696,10 +6723,10 @@
     </row>
     <row r="450" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B450" s="8" t="s">
-        <v>501</v>
+        <v>510</v>
       </c>
       <c r="C450" s="6" t="s">
         <v>119</v>
@@ -6707,10 +6734,10 @@
     </row>
     <row r="451" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B451" s="8" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="C451" s="6" t="s">
         <v>119</v>
@@ -6718,10 +6745,10 @@
     </row>
     <row r="452" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B452" s="8" t="s">
-        <v>503</v>
+        <v>512</v>
       </c>
       <c r="C452" s="6" t="s">
         <v>119</v>
@@ -6729,10 +6756,10 @@
     </row>
     <row r="453" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A453" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B453" s="8" t="s">
-        <v>504</v>
+        <v>513</v>
       </c>
       <c r="C453" s="6" t="s">
         <v>119</v>
@@ -6740,10 +6767,10 @@
     </row>
     <row r="454" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B454" s="8" t="s">
-        <v>505</v>
+        <v>514</v>
       </c>
       <c r="C454" s="6" t="s">
         <v>119</v>
@@ -6751,10 +6778,10 @@
     </row>
     <row r="455" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B455" s="8" t="s">
-        <v>506</v>
+        <v>515</v>
       </c>
       <c r="C455" s="6" t="s">
         <v>119</v>
@@ -6762,10 +6789,10 @@
     </row>
     <row r="456" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B456" s="8" t="s">
-        <v>507</v>
+        <v>516</v>
       </c>
       <c r="C456" s="6" t="s">
         <v>119</v>
@@ -6773,10 +6800,10 @@
     </row>
     <row r="457" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B457" s="8" t="s">
-        <v>508</v>
+        <v>517</v>
       </c>
       <c r="C457" s="6" t="s">
         <v>119</v>
@@ -6784,10 +6811,10 @@
     </row>
     <row r="458" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B458" s="8" t="s">
-        <v>509</v>
+        <v>518</v>
       </c>
       <c r="C458" s="6" t="s">
         <v>119</v>
@@ -6795,10 +6822,10 @@
     </row>
     <row r="459" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A459" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B459" s="8" t="s">
-        <v>510</v>
+        <v>519</v>
       </c>
       <c r="C459" s="6" t="s">
         <v>119</v>
@@ -6806,10 +6833,10 @@
     </row>
     <row r="460" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B460" s="8" t="s">
-        <v>511</v>
+        <v>520</v>
       </c>
       <c r="C460" s="6" t="s">
         <v>119</v>
@@ -6817,10 +6844,10 @@
     </row>
     <row r="461" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B461" s="8" t="s">
-        <v>512</v>
+        <v>521</v>
       </c>
       <c r="C461" s="6" t="s">
         <v>119</v>
@@ -6828,10 +6855,10 @@
     </row>
     <row r="462" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B462" s="8" t="s">
-        <v>513</v>
+        <v>522</v>
       </c>
       <c r="C462" s="6" t="s">
         <v>119</v>
@@ -6839,10 +6866,10 @@
     </row>
     <row r="463" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B463" s="8" t="s">
-        <v>514</v>
+        <v>523</v>
       </c>
       <c r="C463" s="6" t="s">
         <v>119</v>
@@ -6850,10 +6877,10 @@
     </row>
     <row r="464" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B464" s="8" t="s">
-        <v>515</v>
+        <v>524</v>
       </c>
       <c r="C464" s="6" t="s">
         <v>119</v>
@@ -6861,10 +6888,10 @@
     </row>
     <row r="465" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B465" s="8" t="s">
-        <v>516</v>
+        <v>525</v>
       </c>
       <c r="C465" s="6" t="s">
         <v>119</v>
@@ -6872,10 +6899,10 @@
     </row>
     <row r="466" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B466" s="8" t="s">
-        <v>517</v>
+        <v>526</v>
       </c>
       <c r="C466" s="6" t="s">
         <v>119</v>
@@ -6883,10 +6910,10 @@
     </row>
     <row r="467" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B467" s="8" t="s">
-        <v>518</v>
+        <v>527</v>
       </c>
       <c r="C467" s="6" t="s">
         <v>119</v>
@@ -6894,10 +6921,10 @@
     </row>
     <row r="468" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B468" s="8" t="s">
-        <v>519</v>
+        <v>528</v>
       </c>
       <c r="C468" s="6" t="s">
         <v>119</v>
@@ -6905,10 +6932,10 @@
     </row>
     <row r="469" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="7" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
       <c r="B469" s="8" t="s">
-        <v>520</v>
+        <v>529</v>
       </c>
       <c r="C469" s="6" t="s">
         <v>119</v>
@@ -6927,10 +6954,10 @@
     </row>
     <row r="472" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B472" s="8" t="s">
-        <v>522</v>
+        <v>531</v>
       </c>
       <c r="C472" s="6" t="s">
         <v>119</v>
@@ -6938,10 +6965,10 @@
     </row>
     <row r="473" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B473" s="8" t="s">
-        <v>523</v>
+        <v>532</v>
       </c>
       <c r="C473" s="6" t="s">
         <v>119</v>
@@ -6949,10 +6976,10 @@
     </row>
     <row r="474" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B474" s="8" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="C474" s="6" t="s">
         <v>119</v>
@@ -6960,10 +6987,10 @@
     </row>
     <row r="475" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B475" s="8" t="s">
-        <v>525</v>
+        <v>534</v>
       </c>
       <c r="C475" s="6" t="s">
         <v>119</v>
@@ -6971,10 +6998,10 @@
     </row>
     <row r="476" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B476" s="8" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="C476" s="6" t="s">
         <v>119</v>
@@ -6982,10 +7009,10 @@
     </row>
     <row r="477" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B477" s="8" t="s">
-        <v>527</v>
+        <v>536</v>
       </c>
       <c r="C477" s="6" t="s">
         <v>119</v>
@@ -6993,10 +7020,10 @@
     </row>
     <row r="478" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B478" s="8" t="s">
-        <v>528</v>
+        <v>537</v>
       </c>
       <c r="C478" s="6" t="s">
         <v>119</v>
@@ -7004,10 +7031,10 @@
     </row>
     <row r="479" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B479" s="8" t="s">
-        <v>529</v>
+        <v>538</v>
       </c>
       <c r="C479" s="6" t="s">
         <v>119</v>
@@ -7015,10 +7042,10 @@
     </row>
     <row r="480" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B480" s="8" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="C480" s="6" t="s">
         <v>119</v>
@@ -7026,10 +7053,10 @@
     </row>
     <row r="481" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="7" t="s">
-        <v>521</v>
+        <v>530</v>
       </c>
       <c r="B481" s="8" t="s">
-        <v>531</v>
+        <v>540</v>
       </c>
       <c r="C481" s="6" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
Graph added(chinese postman problem incomplete)
</commit_message>
<xml_diff>
--- a/FINAL450.xlsx
+++ b/FINAL450.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="574">
   <si>
     <t xml:space="preserve">YES(Iterative &amp; recursive)</t>
   </si>
@@ -1327,33 +1327,57 @@
     <t xml:space="preserve">Detect Cycle in Directed Graph using BFS/DFS Algo </t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Recall DFS prcedure, BFS Kahn topo sort)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Detect Cycle in UnDirected Graph using BFS/DFS Algo </t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DFS similarPrevious,BFS sameAsBFSalgo)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Search in a Maze</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum Step by Knight</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(BFS and DP)</t>
+  </si>
+  <si>
     <t xml:space="preserve">flood fill algo</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Recursion or BFS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Clone a graph</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DFS/BFS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Making wired Connections</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(BFS/DFS or Union Find)</t>
+  </si>
+  <si>
     <t xml:space="preserve">word Ladder </t>
   </si>
   <si>
+    <t xml:space="preserve">YES(BFS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dijkstra algo</t>
   </si>
   <si>
     <t xml:space="preserve">Implement Topological Sort </t>
   </si>
   <si>
+    <t xml:space="preserve">y(topology sorting Kahn’s Algo)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Minimum time taken by each job to be completed given by a Directed Acyclic Graph</t>
   </si>
   <si>
@@ -1363,18 +1387,33 @@
     <t xml:space="preserve">Find the no. of Isalnds</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(BFS/DFS or Union Find)bfs/dfs faster rn</t>
+  </si>
+  <si>
     <t xml:space="preserve">Given a sorted Dictionary of an Alien Language, find order of characters</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(make adj list and topological sort)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Implement Kruksal’sAlgorithm</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Edge based)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Implement Prim’s Algorithm</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(node based)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total no. of Spanning tree in a graph</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Kirchhoff’s Theorem)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Implement Bellman Ford Algorithm</t>
   </si>
   <si>
@@ -1384,64 +1423,124 @@
     <t xml:space="preserve">Travelling Salesman Problem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(permutation or DP)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Graph ColouringProblem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(recall technique)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Snake and Ladders Problem</t>
   </si>
   <si>
+    <t xml:space="preserve">y(BFS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Find bridge in a graph</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(tough, algo recall)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Count Strongly connected Components(Kosaraju Algo)</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DFS,ReverseGraph,DFS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Check whether a graph is Bipartite or Not</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Graph Coloring)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Detect Negative cycle in a graph</t>
   </si>
   <si>
     <t xml:space="preserve">Longest path in a Directed Acyclic Graph</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(topological order)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Journey to the Moon</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(union find set/DFS to find components)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cheapest Flights Within K Stops</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(Modified Bellman Ford)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Oliver and the Game</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DFS and inTime outTime)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Water Jug problem using BFS</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(3 possible neighbours)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Find if there is a path of more thank length from a source</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DFS and Backtracking)</t>
+  </si>
+  <si>
     <t xml:space="preserve">M-ColouringProblem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(using recursion)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Minimum edges to reverse o make path from source to destination</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(modify graph with reverse edge cost 1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Paths to travel each nodes using each edge(Seven Bridges)</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see method both directed &amp; indirected)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Vertex Cover Problem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(approximate method not actual answer)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chinese Postman or Route Inspection</t>
   </si>
   <si>
+    <t xml:space="preserve">INCOMPLETE</t>
+  </si>
+  <si>
     <t xml:space="preserve">Number of Triangles in a Directed and Undirected Graph</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(count triplet or trace(A^3)/6)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Minimise the cashflow among a given set of friends who have borrowed money from each other</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(recursion give from maxCred to maxDeb)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Two Clique Problem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES(complement and bipartite)</t>
   </si>
   <si>
     <t xml:space="preserve">Trie</t>
@@ -1955,7 +2054,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C481"/>
-  <sheetFormatPr defaultColWidth="8.375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.37890625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.73"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="111.76"/>
@@ -4851,15 +4950,15 @@
       <c r="B274" s="10"/>
       <c r="C274" s="6"/>
     </row>
-    <row r="275" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="7" t="s">
         <v>333</v>
       </c>
       <c r="B275" s="8" t="s">
         <v>334</v>
       </c>
-      <c r="C275" s="6" t="s">
-        <v>119</v>
+      <c r="C275" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="276" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5621,7 +5720,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="347" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="347" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="7" t="s">
         <v>392</v>
       </c>
@@ -5716,8 +5815,8 @@
       <c r="B356" s="8" t="s">
         <v>421</v>
       </c>
-      <c r="C356" s="6" t="s">
-        <v>119</v>
+      <c r="C356" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="357" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5727,96 +5826,96 @@
       <c r="B357" s="8" t="s">
         <v>422</v>
       </c>
-      <c r="C357" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="358" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C357" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="358" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B358" s="8" t="s">
         <v>423</v>
       </c>
-      <c r="C358" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="359" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C358" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="359" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B359" s="8" t="s">
         <v>424</v>
       </c>
-      <c r="C359" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="360" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C359" s="9" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="360" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A360" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B360" s="8" t="s">
-        <v>425</v>
-      </c>
-      <c r="C360" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="361" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>426</v>
+      </c>
+      <c r="C360" s="9" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="361" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B361" s="8" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C361" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="362" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="362" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A362" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B362" s="8" t="s">
-        <v>427</v>
-      </c>
-      <c r="C362" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="363" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>429</v>
+      </c>
+      <c r="C362" s="9" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="363" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B363" s="8" t="s">
-        <v>428</v>
-      </c>
-      <c r="C363" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="364" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>431</v>
+      </c>
+      <c r="C363" s="9" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="364" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B364" s="8" t="s">
-        <v>429</v>
-      </c>
-      <c r="C364" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="365" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>433</v>
+      </c>
+      <c r="C364" s="9" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="365" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B365" s="8" t="s">
-        <v>430</v>
-      </c>
-      <c r="C365" s="6" t="s">
-        <v>119</v>
+        <v>435</v>
+      </c>
+      <c r="C365" s="9" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="366" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5824,153 +5923,153 @@
         <v>420</v>
       </c>
       <c r="B366" s="8" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="C366" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="367" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="367" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B367" s="8" t="s">
-        <v>432</v>
-      </c>
-      <c r="C367" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="368" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>439</v>
+      </c>
+      <c r="C367" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="368" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A368" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B368" s="8" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="C368" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="369" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="369" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A369" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B369" s="8" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="C369" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="370" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="370" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A370" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B370" s="8" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="C370" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="371" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="371" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B371" s="8" t="s">
-        <v>436</v>
-      </c>
-      <c r="C371" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="372" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>444</v>
+      </c>
+      <c r="C371" s="9" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="372" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B372" s="8" t="s">
-        <v>437</v>
-      </c>
-      <c r="C372" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="373" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>446</v>
+      </c>
+      <c r="C372" s="9" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="373" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B373" s="8" t="s">
-        <v>438</v>
-      </c>
-      <c r="C373" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="374" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>448</v>
+      </c>
+      <c r="C373" s="9" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="374" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B374" s="8" t="s">
-        <v>439</v>
-      </c>
-      <c r="C374" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="375" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>450</v>
+      </c>
+      <c r="C374" s="9" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="375" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B375" s="8" t="s">
-        <v>440</v>
-      </c>
-      <c r="C375" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="376" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>452</v>
+      </c>
+      <c r="C375" s="9" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="376" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B376" s="8" t="s">
-        <v>441</v>
-      </c>
-      <c r="C376" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="377" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>454</v>
+      </c>
+      <c r="C376" s="9" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="377" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B377" s="8" t="s">
-        <v>442</v>
-      </c>
-      <c r="C377" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="378" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>455</v>
+      </c>
+      <c r="C377" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="378" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B378" s="8" t="s">
-        <v>443</v>
-      </c>
-      <c r="C378" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="379" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>456</v>
+      </c>
+      <c r="C378" s="9" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="379" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B379" s="8" t="s">
-        <v>444</v>
-      </c>
-      <c r="C379" s="6" t="s">
-        <v>119</v>
+        <v>458</v>
+      </c>
+      <c r="C379" s="9" t="s">
+        <v>459</v>
       </c>
     </row>
     <row r="380" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5978,43 +6077,43 @@
         <v>420</v>
       </c>
       <c r="B380" s="8" t="s">
-        <v>445</v>
+        <v>460</v>
       </c>
       <c r="C380" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="381" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="381" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B381" s="8" t="s">
-        <v>446</v>
-      </c>
-      <c r="C381" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="382" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>462</v>
+      </c>
+      <c r="C381" s="9" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="382" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B382" s="8" t="s">
-        <v>447</v>
-      </c>
-      <c r="C382" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="383" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>464</v>
+      </c>
+      <c r="C382" s="9" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="383" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B383" s="8" t="s">
-        <v>448</v>
-      </c>
-      <c r="C383" s="6" t="s">
-        <v>119</v>
+        <v>466</v>
+      </c>
+      <c r="C383" s="9" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="384" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6022,65 +6121,65 @@
         <v>420</v>
       </c>
       <c r="B384" s="8" t="s">
-        <v>449</v>
+        <v>468</v>
       </c>
       <c r="C384" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="385" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="385" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B385" s="8" t="s">
-        <v>450</v>
-      </c>
-      <c r="C385" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="386" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>469</v>
+      </c>
+      <c r="C385" s="9" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="386" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B386" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="C386" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="387" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>471</v>
+      </c>
+      <c r="C386" s="9" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="387" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B387" s="8" t="s">
-        <v>452</v>
-      </c>
-      <c r="C387" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="388" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>473</v>
+      </c>
+      <c r="C387" s="9" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="388" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B388" s="8" t="s">
-        <v>453</v>
-      </c>
-      <c r="C388" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="389" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>475</v>
+      </c>
+      <c r="C388" s="9" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="389" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B389" s="8" t="s">
-        <v>454</v>
-      </c>
-      <c r="C389" s="6" t="s">
-        <v>119</v>
+        <v>477</v>
+      </c>
+      <c r="C389" s="9" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="390" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6088,109 +6187,109 @@
         <v>420</v>
       </c>
       <c r="B390" s="8" t="s">
-        <v>454</v>
+        <v>477</v>
       </c>
       <c r="C390" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="391" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="391" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B391" s="8" t="s">
-        <v>455</v>
-      </c>
-      <c r="C391" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="392" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>479</v>
+      </c>
+      <c r="C391" s="9" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="392" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B392" s="8" t="s">
-        <v>456</v>
-      </c>
-      <c r="C392" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="393" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>481</v>
+      </c>
+      <c r="C392" s="9" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="393" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B393" s="8" t="s">
-        <v>457</v>
-      </c>
-      <c r="C393" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="394" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>483</v>
+      </c>
+      <c r="C393" s="9" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="394" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B394" s="8" t="s">
-        <v>458</v>
-      </c>
-      <c r="C394" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="395" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>485</v>
+      </c>
+      <c r="C394" s="9" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="395" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B395" s="8" t="s">
-        <v>459</v>
-      </c>
-      <c r="C395" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="396" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>487</v>
+      </c>
+      <c r="C395" s="9" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="396" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B396" s="8" t="s">
-        <v>460</v>
-      </c>
-      <c r="C396" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="397" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>489</v>
+      </c>
+      <c r="C396" s="11" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="397" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B397" s="8" t="s">
-        <v>461</v>
-      </c>
-      <c r="C397" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="398" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>491</v>
+      </c>
+      <c r="C397" s="9" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="398" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B398" s="8" t="s">
-        <v>462</v>
-      </c>
-      <c r="C398" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="399" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>493</v>
+      </c>
+      <c r="C398" s="9" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="399" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="7" t="s">
         <v>420</v>
       </c>
       <c r="B399" s="8" t="s">
-        <v>463</v>
-      </c>
-      <c r="C399" s="6" t="s">
-        <v>119</v>
+        <v>495</v>
+      </c>
+      <c r="C399" s="9" t="s">
+        <v>496</v>
       </c>
     </row>
     <row r="400" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6206,10 +6305,10 @@
     </row>
     <row r="402" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="7" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="B402" s="8" t="s">
-        <v>465</v>
+        <v>498</v>
       </c>
       <c r="C402" s="6" t="s">
         <v>119</v>
@@ -6217,10 +6316,10 @@
     </row>
     <row r="403" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="7" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="B403" s="8" t="s">
-        <v>466</v>
+        <v>499</v>
       </c>
       <c r="C403" s="6" t="s">
         <v>119</v>
@@ -6228,10 +6327,10 @@
     </row>
     <row r="404" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="7" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="B404" s="8" t="s">
-        <v>467</v>
+        <v>500</v>
       </c>
       <c r="C404" s="6" t="s">
         <v>119</v>
@@ -6239,7 +6338,7 @@
     </row>
     <row r="405" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A405" s="7" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="B405" s="8" t="s">
         <v>122</v>
@@ -6250,10 +6349,10 @@
     </row>
     <row r="406" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="7" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="B406" s="8" t="s">
-        <v>468</v>
+        <v>501</v>
       </c>
       <c r="C406" s="6" t="s">
         <v>119</v>
@@ -6261,10 +6360,10 @@
     </row>
     <row r="407" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A407" s="7" t="s">
-        <v>464</v>
+        <v>497</v>
       </c>
       <c r="B407" s="8" t="s">
-        <v>469</v>
+        <v>502</v>
       </c>
       <c r="C407" s="6" t="s">
         <v>119</v>
@@ -6283,10 +6382,10 @@
     </row>
     <row r="410" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B410" s="8" t="s">
-        <v>471</v>
+        <v>504</v>
       </c>
       <c r="C410" s="6" t="s">
         <v>119</v>
@@ -6294,10 +6393,10 @@
     </row>
     <row r="411" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B411" s="8" t="s">
-        <v>472</v>
+        <v>505</v>
       </c>
       <c r="C411" s="6" t="s">
         <v>119</v>
@@ -6305,10 +6404,10 @@
     </row>
     <row r="412" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B412" s="8" t="s">
-        <v>473</v>
+        <v>506</v>
       </c>
       <c r="C412" s="6" t="s">
         <v>119</v>
@@ -6316,10 +6415,10 @@
     </row>
     <row r="413" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>474</v>
+        <v>507</v>
       </c>
       <c r="C413" s="6" t="s">
         <v>119</v>
@@ -6327,10 +6426,10 @@
     </row>
     <row r="414" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>475</v>
+        <v>508</v>
       </c>
       <c r="C414" s="6" t="s">
         <v>119</v>
@@ -6338,10 +6437,10 @@
     </row>
     <row r="415" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B415" s="8" t="s">
-        <v>476</v>
+        <v>509</v>
       </c>
       <c r="C415" s="6" t="s">
         <v>119</v>
@@ -6349,10 +6448,10 @@
     </row>
     <row r="416" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B416" s="8" t="s">
-        <v>477</v>
+        <v>510</v>
       </c>
       <c r="C416" s="6" t="s">
         <v>119</v>
@@ -6360,7 +6459,7 @@
     </row>
     <row r="417" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B417" s="8" t="s">
         <v>341</v>
@@ -6371,10 +6470,10 @@
     </row>
     <row r="418" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B418" s="8" t="s">
-        <v>478</v>
+        <v>511</v>
       </c>
       <c r="C418" s="6" t="s">
         <v>119</v>
@@ -6382,10 +6481,10 @@
     </row>
     <row r="419" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>479</v>
+        <v>512</v>
       </c>
       <c r="C419" s="6" t="s">
         <v>119</v>
@@ -6393,10 +6492,10 @@
     </row>
     <row r="420" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B420" s="8" t="s">
-        <v>480</v>
+        <v>513</v>
       </c>
       <c r="C420" s="6" t="s">
         <v>119</v>
@@ -6404,10 +6503,10 @@
     </row>
     <row r="421" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B421" s="8" t="s">
-        <v>481</v>
+        <v>514</v>
       </c>
       <c r="C421" s="6" t="s">
         <v>119</v>
@@ -6415,10 +6514,10 @@
     </row>
     <row r="422" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>482</v>
+        <v>515</v>
       </c>
       <c r="C422" s="6" t="s">
         <v>119</v>
@@ -6426,10 +6525,10 @@
     </row>
     <row r="423" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B423" s="8" t="s">
-        <v>483</v>
+        <v>516</v>
       </c>
       <c r="C423" s="6" t="s">
         <v>119</v>
@@ -6437,10 +6536,10 @@
     </row>
     <row r="424" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B424" s="8" t="s">
-        <v>484</v>
+        <v>517</v>
       </c>
       <c r="C424" s="6" t="s">
         <v>119</v>
@@ -6448,10 +6547,10 @@
     </row>
     <row r="425" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B425" s="8" t="s">
-        <v>485</v>
+        <v>518</v>
       </c>
       <c r="C425" s="6" t="s">
         <v>119</v>
@@ -6459,10 +6558,10 @@
     </row>
     <row r="426" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B426" s="8" t="s">
-        <v>486</v>
+        <v>519</v>
       </c>
       <c r="C426" s="6" t="s">
         <v>119</v>
@@ -6470,10 +6569,10 @@
     </row>
     <row r="427" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B427" s="8" t="s">
-        <v>487</v>
+        <v>520</v>
       </c>
       <c r="C427" s="6" t="s">
         <v>119</v>
@@ -6481,10 +6580,10 @@
     </row>
     <row r="428" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B428" s="8" t="s">
-        <v>488</v>
+        <v>521</v>
       </c>
       <c r="C428" s="6" t="s">
         <v>119</v>
@@ -6492,10 +6591,10 @@
     </row>
     <row r="429" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B429" s="8" t="s">
-        <v>489</v>
+        <v>522</v>
       </c>
       <c r="C429" s="6" t="s">
         <v>119</v>
@@ -6503,10 +6602,10 @@
     </row>
     <row r="430" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B430" s="8" t="s">
-        <v>490</v>
+        <v>523</v>
       </c>
       <c r="C430" s="6" t="s">
         <v>119</v>
@@ -6514,10 +6613,10 @@
     </row>
     <row r="431" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B431" s="8" t="s">
-        <v>491</v>
+        <v>524</v>
       </c>
       <c r="C431" s="6" t="s">
         <v>119</v>
@@ -6525,10 +6624,10 @@
     </row>
     <row r="432" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B432" s="8" t="s">
-        <v>492</v>
+        <v>525</v>
       </c>
       <c r="C432" s="6" t="s">
         <v>119</v>
@@ -6536,10 +6635,10 @@
     </row>
     <row r="433" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B433" s="8" t="s">
-        <v>493</v>
+        <v>526</v>
       </c>
       <c r="C433" s="6" t="s">
         <v>119</v>
@@ -6547,10 +6646,10 @@
     </row>
     <row r="434" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B434" s="8" t="s">
-        <v>494</v>
+        <v>527</v>
       </c>
       <c r="C434" s="6" t="s">
         <v>119</v>
@@ -6558,10 +6657,10 @@
     </row>
     <row r="435" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A435" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B435" s="8" t="s">
-        <v>495</v>
+        <v>528</v>
       </c>
       <c r="C435" s="6" t="s">
         <v>119</v>
@@ -6569,10 +6668,10 @@
     </row>
     <row r="436" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B436" s="8" t="s">
-        <v>496</v>
+        <v>529</v>
       </c>
       <c r="C436" s="6" t="s">
         <v>119</v>
@@ -6580,10 +6679,10 @@
     </row>
     <row r="437" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B437" s="8" t="s">
-        <v>497</v>
+        <v>530</v>
       </c>
       <c r="C437" s="6" t="s">
         <v>119</v>
@@ -6591,10 +6690,10 @@
     </row>
     <row r="438" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B438" s="8" t="s">
-        <v>498</v>
+        <v>531</v>
       </c>
       <c r="C438" s="6" t="s">
         <v>119</v>
@@ -6602,10 +6701,10 @@
     </row>
     <row r="439" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B439" s="8" t="s">
-        <v>499</v>
+        <v>532</v>
       </c>
       <c r="C439" s="6" t="s">
         <v>119</v>
@@ -6613,10 +6712,10 @@
     </row>
     <row r="440" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B440" s="8" t="s">
-        <v>500</v>
+        <v>533</v>
       </c>
       <c r="C440" s="6" t="s">
         <v>119</v>
@@ -6624,10 +6723,10 @@
     </row>
     <row r="441" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B441" s="8" t="s">
-        <v>501</v>
+        <v>534</v>
       </c>
       <c r="C441" s="6" t="s">
         <v>119</v>
@@ -6635,10 +6734,10 @@
     </row>
     <row r="442" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B442" s="8" t="s">
-        <v>502</v>
+        <v>535</v>
       </c>
       <c r="C442" s="6" t="s">
         <v>119</v>
@@ -6646,10 +6745,10 @@
     </row>
     <row r="443" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B443" s="8" t="s">
-        <v>503</v>
+        <v>536</v>
       </c>
       <c r="C443" s="6" t="s">
         <v>119</v>
@@ -6657,10 +6756,10 @@
     </row>
     <row r="444" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B444" s="8" t="s">
-        <v>504</v>
+        <v>537</v>
       </c>
       <c r="C444" s="6" t="s">
         <v>119</v>
@@ -6668,10 +6767,10 @@
     </row>
     <row r="445" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B445" s="8" t="s">
-        <v>505</v>
+        <v>538</v>
       </c>
       <c r="C445" s="6" t="s">
         <v>119</v>
@@ -6679,10 +6778,10 @@
     </row>
     <row r="446" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B446" s="8" t="s">
-        <v>506</v>
+        <v>539</v>
       </c>
       <c r="C446" s="6" t="s">
         <v>119</v>
@@ -6690,10 +6789,10 @@
     </row>
     <row r="447" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B447" s="8" t="s">
-        <v>507</v>
+        <v>540</v>
       </c>
       <c r="C447" s="6" t="s">
         <v>119</v>
@@ -6701,10 +6800,10 @@
     </row>
     <row r="448" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B448" s="8" t="s">
-        <v>508</v>
+        <v>541</v>
       </c>
       <c r="C448" s="6" t="s">
         <v>119</v>
@@ -6712,10 +6811,10 @@
     </row>
     <row r="449" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B449" s="8" t="s">
-        <v>509</v>
+        <v>542</v>
       </c>
       <c r="C449" s="6" t="s">
         <v>119</v>
@@ -6723,10 +6822,10 @@
     </row>
     <row r="450" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B450" s="8" t="s">
-        <v>510</v>
+        <v>543</v>
       </c>
       <c r="C450" s="6" t="s">
         <v>119</v>
@@ -6734,10 +6833,10 @@
     </row>
     <row r="451" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B451" s="8" t="s">
-        <v>511</v>
+        <v>544</v>
       </c>
       <c r="C451" s="6" t="s">
         <v>119</v>
@@ -6745,10 +6844,10 @@
     </row>
     <row r="452" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B452" s="8" t="s">
-        <v>512</v>
+        <v>545</v>
       </c>
       <c r="C452" s="6" t="s">
         <v>119</v>
@@ -6756,10 +6855,10 @@
     </row>
     <row r="453" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A453" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B453" s="8" t="s">
-        <v>513</v>
+        <v>546</v>
       </c>
       <c r="C453" s="6" t="s">
         <v>119</v>
@@ -6767,10 +6866,10 @@
     </row>
     <row r="454" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B454" s="8" t="s">
-        <v>514</v>
+        <v>547</v>
       </c>
       <c r="C454" s="6" t="s">
         <v>119</v>
@@ -6778,10 +6877,10 @@
     </row>
     <row r="455" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B455" s="8" t="s">
-        <v>515</v>
+        <v>548</v>
       </c>
       <c r="C455" s="6" t="s">
         <v>119</v>
@@ -6789,10 +6888,10 @@
     </row>
     <row r="456" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B456" s="8" t="s">
-        <v>516</v>
+        <v>549</v>
       </c>
       <c r="C456" s="6" t="s">
         <v>119</v>
@@ -6800,10 +6899,10 @@
     </row>
     <row r="457" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B457" s="8" t="s">
-        <v>517</v>
+        <v>550</v>
       </c>
       <c r="C457" s="6" t="s">
         <v>119</v>
@@ -6811,10 +6910,10 @@
     </row>
     <row r="458" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B458" s="8" t="s">
-        <v>518</v>
+        <v>551</v>
       </c>
       <c r="C458" s="6" t="s">
         <v>119</v>
@@ -6822,10 +6921,10 @@
     </row>
     <row r="459" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A459" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B459" s="8" t="s">
-        <v>519</v>
+        <v>552</v>
       </c>
       <c r="C459" s="6" t="s">
         <v>119</v>
@@ -6833,10 +6932,10 @@
     </row>
     <row r="460" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B460" s="8" t="s">
-        <v>520</v>
+        <v>553</v>
       </c>
       <c r="C460" s="6" t="s">
         <v>119</v>
@@ -6844,10 +6943,10 @@
     </row>
     <row r="461" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B461" s="8" t="s">
-        <v>521</v>
+        <v>554</v>
       </c>
       <c r="C461" s="6" t="s">
         <v>119</v>
@@ -6855,10 +6954,10 @@
     </row>
     <row r="462" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B462" s="8" t="s">
-        <v>522</v>
+        <v>555</v>
       </c>
       <c r="C462" s="6" t="s">
         <v>119</v>
@@ -6866,10 +6965,10 @@
     </row>
     <row r="463" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B463" s="8" t="s">
-        <v>523</v>
+        <v>556</v>
       </c>
       <c r="C463" s="6" t="s">
         <v>119</v>
@@ -6877,10 +6976,10 @@
     </row>
     <row r="464" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B464" s="8" t="s">
-        <v>524</v>
+        <v>557</v>
       </c>
       <c r="C464" s="6" t="s">
         <v>119</v>
@@ -6888,10 +6987,10 @@
     </row>
     <row r="465" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B465" s="8" t="s">
-        <v>525</v>
+        <v>558</v>
       </c>
       <c r="C465" s="6" t="s">
         <v>119</v>
@@ -6899,10 +6998,10 @@
     </row>
     <row r="466" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B466" s="8" t="s">
-        <v>526</v>
+        <v>559</v>
       </c>
       <c r="C466" s="6" t="s">
         <v>119</v>
@@ -6910,10 +7009,10 @@
     </row>
     <row r="467" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B467" s="8" t="s">
-        <v>527</v>
+        <v>560</v>
       </c>
       <c r="C467" s="6" t="s">
         <v>119</v>
@@ -6921,10 +7020,10 @@
     </row>
     <row r="468" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B468" s="8" t="s">
-        <v>528</v>
+        <v>561</v>
       </c>
       <c r="C468" s="6" t="s">
         <v>119</v>
@@ -6932,10 +7031,10 @@
     </row>
     <row r="469" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="7" t="s">
-        <v>470</v>
+        <v>503</v>
       </c>
       <c r="B469" s="8" t="s">
-        <v>529</v>
+        <v>562</v>
       </c>
       <c r="C469" s="6" t="s">
         <v>119</v>
@@ -6954,10 +7053,10 @@
     </row>
     <row r="472" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B472" s="8" t="s">
-        <v>531</v>
+        <v>564</v>
       </c>
       <c r="C472" s="6" t="s">
         <v>119</v>
@@ -6965,10 +7064,10 @@
     </row>
     <row r="473" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B473" s="8" t="s">
-        <v>532</v>
+        <v>565</v>
       </c>
       <c r="C473" s="6" t="s">
         <v>119</v>
@@ -6976,10 +7075,10 @@
     </row>
     <row r="474" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B474" s="8" t="s">
-        <v>533</v>
+        <v>566</v>
       </c>
       <c r="C474" s="6" t="s">
         <v>119</v>
@@ -6987,10 +7086,10 @@
     </row>
     <row r="475" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B475" s="8" t="s">
-        <v>534</v>
+        <v>567</v>
       </c>
       <c r="C475" s="6" t="s">
         <v>119</v>
@@ -6998,10 +7097,10 @@
     </row>
     <row r="476" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B476" s="8" t="s">
-        <v>535</v>
+        <v>568</v>
       </c>
       <c r="C476" s="6" t="s">
         <v>119</v>
@@ -7009,10 +7108,10 @@
     </row>
     <row r="477" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B477" s="8" t="s">
-        <v>536</v>
+        <v>569</v>
       </c>
       <c r="C477" s="6" t="s">
         <v>119</v>
@@ -7020,10 +7119,10 @@
     </row>
     <row r="478" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B478" s="8" t="s">
-        <v>537</v>
+        <v>570</v>
       </c>
       <c r="C478" s="6" t="s">
         <v>119</v>
@@ -7031,10 +7130,10 @@
     </row>
     <row r="479" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B479" s="8" t="s">
-        <v>538</v>
+        <v>571</v>
       </c>
       <c r="C479" s="6" t="s">
         <v>119</v>
@@ -7042,10 +7141,10 @@
     </row>
     <row r="480" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B480" s="8" t="s">
-        <v>539</v>
+        <v>572</v>
       </c>
       <c r="C480" s="6" t="s">
         <v>119</v>
@@ -7053,10 +7152,10 @@
     </row>
     <row r="481" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="7" t="s">
-        <v>530</v>
+        <v>563</v>
       </c>
       <c r="B481" s="8" t="s">
-        <v>540</v>
+        <v>573</v>
       </c>
       <c r="C481" s="6" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
Trie added and optimized method added in string's 36th question
</commit_message>
<xml_diff>
--- a/FINAL450.xlsx
+++ b/FINAL450.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="580">
   <si>
     <t xml:space="preserve">YES(Iterative &amp; recursive)</t>
   </si>
@@ -1549,16 +1549,34 @@
     <t xml:space="preserve">Construct a trie from scratch</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(insertion,searching,deleting)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Find shortest unique prefix for every word in a given list</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(frequency)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Word Break Problem | (Trie solution)</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(trie+memoization)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES(sort &amp; insert into trie store word in leaf vector)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Implement a Phone Directory</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DFS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Print unique rows in a given boolean matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES(check while insertion)</t>
   </si>
   <si>
     <t xml:space="preserve">Dynamic Programming</t>
@@ -6303,15 +6321,15 @@
       <c r="B401" s="10"/>
       <c r="C401" s="6"/>
     </row>
-    <row r="402" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="402" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="7" t="s">
         <v>497</v>
       </c>
       <c r="B402" s="8" t="s">
         <v>498</v>
       </c>
-      <c r="C402" s="6" t="s">
-        <v>119</v>
+      <c r="C402" s="9" t="s">
+        <v>499</v>
       </c>
     </row>
     <row r="403" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6319,10 +6337,10 @@
         <v>497</v>
       </c>
       <c r="B403" s="8" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="C403" s="6" t="s">
-        <v>119</v>
+        <v>501</v>
       </c>
     </row>
     <row r="404" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6330,10 +6348,10 @@
         <v>497</v>
       </c>
       <c r="B404" s="8" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C404" s="6" t="s">
-        <v>119</v>
+        <v>503</v>
       </c>
     </row>
     <row r="405" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6344,18 +6362,18 @@
         <v>122</v>
       </c>
       <c r="C405" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="406" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="406" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="7" t="s">
         <v>497</v>
       </c>
       <c r="B406" s="8" t="s">
-        <v>501</v>
-      </c>
-      <c r="C406" s="6" t="s">
-        <v>119</v>
+        <v>505</v>
+      </c>
+      <c r="C406" s="9" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="407" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6363,10 +6381,10 @@
         <v>497</v>
       </c>
       <c r="B407" s="8" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="C407" s="6" t="s">
-        <v>119</v>
+        <v>508</v>
       </c>
     </row>
     <row r="408" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6382,10 +6400,10 @@
     </row>
     <row r="410" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B410" s="8" t="s">
-        <v>504</v>
+        <v>510</v>
       </c>
       <c r="C410" s="6" t="s">
         <v>119</v>
@@ -6393,10 +6411,10 @@
     </row>
     <row r="411" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B411" s="8" t="s">
-        <v>505</v>
+        <v>511</v>
       </c>
       <c r="C411" s="6" t="s">
         <v>119</v>
@@ -6404,10 +6422,10 @@
     </row>
     <row r="412" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B412" s="8" t="s">
-        <v>506</v>
+        <v>512</v>
       </c>
       <c r="C412" s="6" t="s">
         <v>119</v>
@@ -6415,10 +6433,10 @@
     </row>
     <row r="413" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="C413" s="6" t="s">
         <v>119</v>
@@ -6426,10 +6444,10 @@
     </row>
     <row r="414" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="C414" s="6" t="s">
         <v>119</v>
@@ -6437,10 +6455,10 @@
     </row>
     <row r="415" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B415" s="8" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="C415" s="6" t="s">
         <v>119</v>
@@ -6448,10 +6466,10 @@
     </row>
     <row r="416" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B416" s="8" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="C416" s="6" t="s">
         <v>119</v>
@@ -6459,7 +6477,7 @@
     </row>
     <row r="417" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B417" s="8" t="s">
         <v>341</v>
@@ -6470,10 +6488,10 @@
     </row>
     <row r="418" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B418" s="8" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C418" s="6" t="s">
         <v>119</v>
@@ -6481,10 +6499,10 @@
     </row>
     <row r="419" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A419" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>512</v>
+        <v>518</v>
       </c>
       <c r="C419" s="6" t="s">
         <v>119</v>
@@ -6492,10 +6510,10 @@
     </row>
     <row r="420" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A420" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B420" s="8" t="s">
-        <v>513</v>
+        <v>519</v>
       </c>
       <c r="C420" s="6" t="s">
         <v>119</v>
@@ -6503,10 +6521,10 @@
     </row>
     <row r="421" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A421" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B421" s="8" t="s">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="C421" s="6" t="s">
         <v>119</v>
@@ -6514,10 +6532,10 @@
     </row>
     <row r="422" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A422" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>515</v>
+        <v>521</v>
       </c>
       <c r="C422" s="6" t="s">
         <v>119</v>
@@ -6525,10 +6543,10 @@
     </row>
     <row r="423" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A423" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B423" s="8" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="C423" s="6" t="s">
         <v>119</v>
@@ -6536,10 +6554,10 @@
     </row>
     <row r="424" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A424" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B424" s="8" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="C424" s="6" t="s">
         <v>119</v>
@@ -6547,10 +6565,10 @@
     </row>
     <row r="425" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B425" s="8" t="s">
-        <v>518</v>
+        <v>524</v>
       </c>
       <c r="C425" s="6" t="s">
         <v>119</v>
@@ -6558,10 +6576,10 @@
     </row>
     <row r="426" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A426" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B426" s="8" t="s">
-        <v>519</v>
+        <v>525</v>
       </c>
       <c r="C426" s="6" t="s">
         <v>119</v>
@@ -6569,10 +6587,10 @@
     </row>
     <row r="427" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A427" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B427" s="8" t="s">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="C427" s="6" t="s">
         <v>119</v>
@@ -6580,10 +6598,10 @@
     </row>
     <row r="428" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A428" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B428" s="8" t="s">
-        <v>521</v>
+        <v>527</v>
       </c>
       <c r="C428" s="6" t="s">
         <v>119</v>
@@ -6591,10 +6609,10 @@
     </row>
     <row r="429" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A429" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B429" s="8" t="s">
-        <v>522</v>
+        <v>528</v>
       </c>
       <c r="C429" s="6" t="s">
         <v>119</v>
@@ -6602,10 +6620,10 @@
     </row>
     <row r="430" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A430" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B430" s="8" t="s">
-        <v>523</v>
+        <v>529</v>
       </c>
       <c r="C430" s="6" t="s">
         <v>119</v>
@@ -6613,10 +6631,10 @@
     </row>
     <row r="431" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B431" s="8" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="C431" s="6" t="s">
         <v>119</v>
@@ -6624,10 +6642,10 @@
     </row>
     <row r="432" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B432" s="8" t="s">
-        <v>525</v>
+        <v>531</v>
       </c>
       <c r="C432" s="6" t="s">
         <v>119</v>
@@ -6635,10 +6653,10 @@
     </row>
     <row r="433" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B433" s="8" t="s">
-        <v>526</v>
+        <v>532</v>
       </c>
       <c r="C433" s="6" t="s">
         <v>119</v>
@@ -6646,10 +6664,10 @@
     </row>
     <row r="434" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B434" s="8" t="s">
-        <v>527</v>
+        <v>533</v>
       </c>
       <c r="C434" s="6" t="s">
         <v>119</v>
@@ -6657,10 +6675,10 @@
     </row>
     <row r="435" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A435" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B435" s="8" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="C435" s="6" t="s">
         <v>119</v>
@@ -6668,10 +6686,10 @@
     </row>
     <row r="436" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B436" s="8" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="C436" s="6" t="s">
         <v>119</v>
@@ -6679,10 +6697,10 @@
     </row>
     <row r="437" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B437" s="8" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="C437" s="6" t="s">
         <v>119</v>
@@ -6690,10 +6708,10 @@
     </row>
     <row r="438" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B438" s="8" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="C438" s="6" t="s">
         <v>119</v>
@@ -6701,10 +6719,10 @@
     </row>
     <row r="439" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A439" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B439" s="8" t="s">
-        <v>532</v>
+        <v>538</v>
       </c>
       <c r="C439" s="6" t="s">
         <v>119</v>
@@ -6712,10 +6730,10 @@
     </row>
     <row r="440" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B440" s="8" t="s">
-        <v>533</v>
+        <v>539</v>
       </c>
       <c r="C440" s="6" t="s">
         <v>119</v>
@@ -6723,10 +6741,10 @@
     </row>
     <row r="441" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A441" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B441" s="8" t="s">
-        <v>534</v>
+        <v>540</v>
       </c>
       <c r="C441" s="6" t="s">
         <v>119</v>
@@ -6734,10 +6752,10 @@
     </row>
     <row r="442" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A442" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B442" s="8" t="s">
-        <v>535</v>
+        <v>541</v>
       </c>
       <c r="C442" s="6" t="s">
         <v>119</v>
@@ -6745,10 +6763,10 @@
     </row>
     <row r="443" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B443" s="8" t="s">
-        <v>536</v>
+        <v>542</v>
       </c>
       <c r="C443" s="6" t="s">
         <v>119</v>
@@ -6756,10 +6774,10 @@
     </row>
     <row r="444" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B444" s="8" t="s">
-        <v>537</v>
+        <v>543</v>
       </c>
       <c r="C444" s="6" t="s">
         <v>119</v>
@@ -6767,10 +6785,10 @@
     </row>
     <row r="445" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B445" s="8" t="s">
-        <v>538</v>
+        <v>544</v>
       </c>
       <c r="C445" s="6" t="s">
         <v>119</v>
@@ -6778,10 +6796,10 @@
     </row>
     <row r="446" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B446" s="8" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="C446" s="6" t="s">
         <v>119</v>
@@ -6789,10 +6807,10 @@
     </row>
     <row r="447" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B447" s="8" t="s">
-        <v>540</v>
+        <v>546</v>
       </c>
       <c r="C447" s="6" t="s">
         <v>119</v>
@@ -6800,10 +6818,10 @@
     </row>
     <row r="448" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B448" s="8" t="s">
-        <v>541</v>
+        <v>547</v>
       </c>
       <c r="C448" s="6" t="s">
         <v>119</v>
@@ -6811,10 +6829,10 @@
     </row>
     <row r="449" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B449" s="8" t="s">
-        <v>542</v>
+        <v>548</v>
       </c>
       <c r="C449" s="6" t="s">
         <v>119</v>
@@ -6822,10 +6840,10 @@
     </row>
     <row r="450" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A450" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B450" s="8" t="s">
-        <v>543</v>
+        <v>549</v>
       </c>
       <c r="C450" s="6" t="s">
         <v>119</v>
@@ -6833,10 +6851,10 @@
     </row>
     <row r="451" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B451" s="8" t="s">
-        <v>544</v>
+        <v>550</v>
       </c>
       <c r="C451" s="6" t="s">
         <v>119</v>
@@ -6844,10 +6862,10 @@
     </row>
     <row r="452" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A452" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B452" s="8" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="C452" s="6" t="s">
         <v>119</v>
@@ -6855,10 +6873,10 @@
     </row>
     <row r="453" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A453" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B453" s="8" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="C453" s="6" t="s">
         <v>119</v>
@@ -6866,10 +6884,10 @@
     </row>
     <row r="454" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B454" s="8" t="s">
-        <v>547</v>
+        <v>553</v>
       </c>
       <c r="C454" s="6" t="s">
         <v>119</v>
@@ -6877,10 +6895,10 @@
     </row>
     <row r="455" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B455" s="8" t="s">
-        <v>548</v>
+        <v>554</v>
       </c>
       <c r="C455" s="6" t="s">
         <v>119</v>
@@ -6888,10 +6906,10 @@
     </row>
     <row r="456" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A456" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B456" s="8" t="s">
-        <v>549</v>
+        <v>555</v>
       </c>
       <c r="C456" s="6" t="s">
         <v>119</v>
@@ -6899,10 +6917,10 @@
     </row>
     <row r="457" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A457" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B457" s="8" t="s">
-        <v>550</v>
+        <v>556</v>
       </c>
       <c r="C457" s="6" t="s">
         <v>119</v>
@@ -6910,10 +6928,10 @@
     </row>
     <row r="458" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A458" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B458" s="8" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="C458" s="6" t="s">
         <v>119</v>
@@ -6921,10 +6939,10 @@
     </row>
     <row r="459" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A459" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B459" s="8" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="C459" s="6" t="s">
         <v>119</v>
@@ -6932,10 +6950,10 @@
     </row>
     <row r="460" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B460" s="8" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="C460" s="6" t="s">
         <v>119</v>
@@ -6943,10 +6961,10 @@
     </row>
     <row r="461" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B461" s="8" t="s">
-        <v>554</v>
+        <v>560</v>
       </c>
       <c r="C461" s="6" t="s">
         <v>119</v>
@@ -6954,10 +6972,10 @@
     </row>
     <row r="462" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B462" s="8" t="s">
-        <v>555</v>
+        <v>561</v>
       </c>
       <c r="C462" s="6" t="s">
         <v>119</v>
@@ -6965,10 +6983,10 @@
     </row>
     <row r="463" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A463" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B463" s="8" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="C463" s="6" t="s">
         <v>119</v>
@@ -6976,10 +6994,10 @@
     </row>
     <row r="464" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A464" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B464" s="8" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="C464" s="6" t="s">
         <v>119</v>
@@ -6987,10 +7005,10 @@
     </row>
     <row r="465" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B465" s="8" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="C465" s="6" t="s">
         <v>119</v>
@@ -6998,10 +7016,10 @@
     </row>
     <row r="466" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A466" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B466" s="8" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="C466" s="6" t="s">
         <v>119</v>
@@ -7009,10 +7027,10 @@
     </row>
     <row r="467" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A467" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B467" s="8" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="C467" s="6" t="s">
         <v>119</v>
@@ -7020,10 +7038,10 @@
     </row>
     <row r="468" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A468" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B468" s="8" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="C468" s="6" t="s">
         <v>119</v>
@@ -7031,10 +7049,10 @@
     </row>
     <row r="469" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A469" s="7" t="s">
-        <v>503</v>
+        <v>509</v>
       </c>
       <c r="B469" s="8" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="C469" s="6" t="s">
         <v>119</v>
@@ -7053,10 +7071,10 @@
     </row>
     <row r="472" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B472" s="8" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="C472" s="6" t="s">
         <v>119</v>
@@ -7064,10 +7082,10 @@
     </row>
     <row r="473" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B473" s="8" t="s">
-        <v>565</v>
+        <v>571</v>
       </c>
       <c r="C473" s="6" t="s">
         <v>119</v>
@@ -7075,10 +7093,10 @@
     </row>
     <row r="474" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B474" s="8" t="s">
-        <v>566</v>
+        <v>572</v>
       </c>
       <c r="C474" s="6" t="s">
         <v>119</v>
@@ -7086,10 +7104,10 @@
     </row>
     <row r="475" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B475" s="8" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="C475" s="6" t="s">
         <v>119</v>
@@ -7097,10 +7115,10 @@
     </row>
     <row r="476" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B476" s="8" t="s">
-        <v>568</v>
+        <v>574</v>
       </c>
       <c r="C476" s="6" t="s">
         <v>119</v>
@@ -7108,10 +7126,10 @@
     </row>
     <row r="477" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B477" s="8" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="C477" s="6" t="s">
         <v>119</v>
@@ -7119,10 +7137,10 @@
     </row>
     <row r="478" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B478" s="8" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="C478" s="6" t="s">
         <v>119</v>
@@ -7130,10 +7148,10 @@
     </row>
     <row r="479" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B479" s="8" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="C479" s="6" t="s">
         <v>119</v>
@@ -7141,10 +7159,10 @@
     </row>
     <row r="480" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B480" s="8" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="C480" s="6" t="s">
         <v>119</v>
@@ -7152,10 +7170,10 @@
     </row>
     <row r="481" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="7" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="B481" s="8" t="s">
-        <v>573</v>
+        <v>579</v>
       </c>
       <c r="C481" s="6" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
New Temp dp incomplete array 25th altered
</commit_message>
<xml_diff>
--- a/FINAL450.xlsx
+++ b/FINAL450.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="613">
   <si>
     <t xml:space="preserve">YES(Iterative &amp; recursive)</t>
   </si>
@@ -1612,21 +1612,36 @@
     <t xml:space="preserve">Binomial CoefficientProblem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see subproblem formulae of nCr)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Permutation CoefficientProblem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see subproblem formulae of nPr)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Program for nth Catalan Number</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see catalan series formation)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Matrix Chain Multiplication </t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see the indexing part)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Edit Distance</t>
   </si>
   <si>
     <t xml:space="preserve">Friends Pairing Problem</t>
   </si>
   <si>
+    <t xml:space="preserve">y(see formulae)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gold Mine Problem</t>
   </si>
   <si>
@@ -1636,6 +1651,9 @@
     <t xml:space="preserve">Painting the Fenceproblem</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see formulae)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximize The Cut Segments</t>
   </si>
   <si>
@@ -1648,21 +1666,36 @@
     <t xml:space="preserve">Longest Increasing Subsequence</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(using LCS concept OR binary search to find length)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Space Optimized Solution of LCS</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see 0/1 alternating procedure of indexing)</t>
+  </si>
+  <si>
     <t xml:space="preserve">LCS (Longest Common Subsequence) of three strings</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(using extended LCS on three arrays)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum Sum Increasing Subsequence</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(LIS for sum instead of length)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Count all subsequences having product less than K</t>
   </si>
   <si>
     <t xml:space="preserve">Longest subsequence such that difference between adjacent is one</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(LIS)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum subsequence sum such that no three are consecutive</t>
   </si>
   <si>
@@ -1672,13 +1705,19 @@
     <t xml:space="preserve">Maximum Length Chain of Pairs</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(LIS after sorting)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum size square sub-matrix with all 1s</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(See algorithm)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Maximum sum of pairs with specific difference</t>
   </si>
   <si>
-    <t xml:space="preserve">Min Cost PathProblem</t>
+    <t xml:space="preserve">Max Cost PathProblem</t>
   </si>
   <si>
     <t xml:space="preserve">Maximum difference of zeros and ones in binary string</t>
@@ -1687,18 +1726,27 @@
     <t xml:space="preserve">Minimum number of jumps to reach end</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(See O(n) solution carefully)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Minimum cost to fill given weight in a bag</t>
   </si>
   <si>
     <t xml:space="preserve">Minimum removals from array to make max –min &lt;= K</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(DP or Binary Search)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Longest Common Substring</t>
   </si>
   <si>
     <t xml:space="preserve">Count number of ways to reacha given score in a game</t>
   </si>
   <si>
+    <t xml:space="preserve">y(count ways of coin change)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Count Balanced Binary Trees of Height h</t>
   </si>
   <si>
@@ -1708,12 +1756,18 @@
     <t xml:space="preserve">Smallest sum contiguous subarray</t>
   </si>
   <si>
+    <t xml:space="preserve">y(same as above just find min instead)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Unbounded Knapsack (Repetition of items allowed)</t>
   </si>
   <si>
     <t xml:space="preserve">Word Break Problem</t>
   </si>
   <si>
+    <t xml:space="preserve">y(used trie for dictionary)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Largest Independent Set Problem</t>
   </si>
   <si>
@@ -1726,13 +1780,25 @@
     <t xml:space="preserve">Count All Palindromic Subsequence in a given String</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(non distinct part is messy just keep in mind)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Longest Palindromic Substring</t>
   </si>
   <si>
+    <t xml:space="preserve">y(similar as above)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Longest alternating subsequence</t>
   </si>
   <si>
+    <t xml:space="preserve">YES(see O(n) approach similar to O(n^2)(LIS))</t>
+  </si>
+  <si>
     <t xml:space="preserve">Weighted Job Scheduling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES(LIS method also used check it something’s faulty)</t>
   </si>
   <si>
     <t xml:space="preserve">Coin game winner where every player has three choices</t>
@@ -2105,11 +2171,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C481"/>
-  <sheetFormatPr defaultColWidth="8.41796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="111.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="49.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="126.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="51.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="4" style="0" width="11.51"/>
   </cols>
   <sheetData>
@@ -5001,7 +5067,7 @@
       <c r="B274" s="10"/>
       <c r="C274" s="6"/>
     </row>
-    <row r="275" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A275" s="7" t="s">
         <v>333</v>
       </c>
@@ -5012,7 +5078,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="276" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A276" s="7" t="s">
         <v>333</v>
       </c>
@@ -5034,7 +5100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="278" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A278" s="7" t="s">
         <v>333</v>
       </c>
@@ -5045,7 +5111,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="279" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="279" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A279" s="7" t="s">
         <v>333</v>
       </c>
@@ -5056,7 +5122,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="280" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A280" s="7" t="s">
         <v>333</v>
       </c>
@@ -5067,7 +5133,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="281" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A281" s="7" t="s">
         <v>333</v>
       </c>
@@ -5089,7 +5155,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="s">
         <v>333</v>
       </c>
@@ -5100,7 +5166,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="284" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="7" t="s">
         <v>333</v>
       </c>
@@ -5111,7 +5177,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="7" t="s">
         <v>333</v>
       </c>
@@ -5133,7 +5199,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="287" customFormat="false" ht="21.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="7" t="s">
         <v>333</v>
       </c>
@@ -5188,7 +5254,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="21.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="7" t="s">
         <v>333</v>
       </c>
@@ -5199,7 +5265,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="293" customFormat="false" ht="21.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A293" s="7" t="s">
         <v>333</v>
       </c>
@@ -5881,7 +5947,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="358" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="358" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="7" t="s">
         <v>427</v>
       </c>
@@ -5892,7 +5958,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="359" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="359" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A359" s="7" t="s">
         <v>427</v>
       </c>
@@ -5903,7 +5969,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="360" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="360" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A360" s="7" t="s">
         <v>427</v>
       </c>
@@ -5914,7 +5980,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="361" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="361" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="7" t="s">
         <v>427</v>
       </c>
@@ -5925,7 +5991,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="362" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="362" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A362" s="7" t="s">
         <v>427</v>
       </c>
@@ -5936,7 +6002,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="363" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="363" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A363" s="7" t="s">
         <v>427</v>
       </c>
@@ -5947,7 +6013,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="364" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="364" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A364" s="7" t="s">
         <v>427</v>
       </c>
@@ -5958,7 +6024,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="365" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="365" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="7" t="s">
         <v>427</v>
       </c>
@@ -5980,7 +6046,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="367" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="367" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="7" t="s">
         <v>427</v>
       </c>
@@ -5991,7 +6057,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="368" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="368" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A368" s="7" t="s">
         <v>427</v>
       </c>
@@ -6002,7 +6068,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="369" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="369" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A369" s="7" t="s">
         <v>427</v>
       </c>
@@ -6013,7 +6079,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="370" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="370" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A370" s="7" t="s">
         <v>427</v>
       </c>
@@ -6024,7 +6090,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="371" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="371" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="7" t="s">
         <v>427</v>
       </c>
@@ -6035,7 +6101,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="372" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="372" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="7" t="s">
         <v>427</v>
       </c>
@@ -6046,7 +6112,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="373" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="373" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A373" s="7" t="s">
         <v>427</v>
       </c>
@@ -6057,7 +6123,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="374" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="374" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="7" t="s">
         <v>427</v>
       </c>
@@ -6068,7 +6134,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="375" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="375" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A375" s="7" t="s">
         <v>427</v>
       </c>
@@ -6079,7 +6145,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="376" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="376" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="7" t="s">
         <v>427</v>
       </c>
@@ -6090,7 +6156,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="377" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="377" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A377" s="7" t="s">
         <v>427</v>
       </c>
@@ -6101,7 +6167,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="378" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="378" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A378" s="7" t="s">
         <v>427</v>
       </c>
@@ -6112,7 +6178,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="379" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="379" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A379" s="7" t="s">
         <v>427</v>
       </c>
@@ -6134,7 +6200,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="381" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="381" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="7" t="s">
         <v>427</v>
       </c>
@@ -6145,7 +6211,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="382" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="382" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A382" s="7" t="s">
         <v>427</v>
       </c>
@@ -6156,7 +6222,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="383" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="383" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A383" s="7" t="s">
         <v>427</v>
       </c>
@@ -6178,7 +6244,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="385" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="385" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="7" t="s">
         <v>427</v>
       </c>
@@ -6189,7 +6255,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="386" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="386" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="7" t="s">
         <v>427</v>
       </c>
@@ -6200,7 +6266,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="387" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="387" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="7" t="s">
         <v>427</v>
       </c>
@@ -6211,7 +6277,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="388" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="388" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="7" t="s">
         <v>427</v>
       </c>
@@ -6222,7 +6288,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="389" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="389" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="7" t="s">
         <v>427</v>
       </c>
@@ -6244,7 +6310,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="391" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="391" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="7" t="s">
         <v>427</v>
       </c>
@@ -6255,7 +6321,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="392" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="392" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="7" t="s">
         <v>427</v>
       </c>
@@ -6266,7 +6332,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="393" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="393" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="7" t="s">
         <v>427</v>
       </c>
@@ -6277,7 +6343,7 @@
         <v>491</v>
       </c>
     </row>
-    <row r="394" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="394" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="7" t="s">
         <v>427</v>
       </c>
@@ -6288,7 +6354,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="395" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="395" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="7" t="s">
         <v>427</v>
       </c>
@@ -6299,7 +6365,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="396" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="396" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="7" t="s">
         <v>427</v>
       </c>
@@ -6310,7 +6376,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="397" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="397" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="7" t="s">
         <v>427</v>
       </c>
@@ -6321,7 +6387,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="398" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="398" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="7" t="s">
         <v>427</v>
       </c>
@@ -6332,7 +6398,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="399" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="399" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="7" t="s">
         <v>427</v>
       </c>
@@ -6354,7 +6420,7 @@
       <c r="B401" s="10"/>
       <c r="C401" s="6"/>
     </row>
-    <row r="402" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="402" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="7" t="s">
         <v>504</v>
       </c>
@@ -6398,7 +6464,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="406" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="406" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A406" s="7" t="s">
         <v>504</v>
       </c>
@@ -6439,7 +6505,7 @@
         <v>517</v>
       </c>
       <c r="C410" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="411" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6450,7 +6516,7 @@
         <v>518</v>
       </c>
       <c r="C411" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="412" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6461,7 +6527,7 @@
         <v>519</v>
       </c>
       <c r="C412" s="6" t="s">
-        <v>119</v>
+        <v>520</v>
       </c>
     </row>
     <row r="413" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6469,10 +6535,10 @@
         <v>516</v>
       </c>
       <c r="B413" s="8" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="C413" s="6" t="s">
-        <v>119</v>
+        <v>522</v>
       </c>
     </row>
     <row r="414" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6480,10 +6546,10 @@
         <v>516</v>
       </c>
       <c r="B414" s="8" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C414" s="6" t="s">
-        <v>119</v>
+        <v>524</v>
       </c>
     </row>
     <row r="415" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6491,10 +6557,10 @@
         <v>516</v>
       </c>
       <c r="B415" s="8" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="C415" s="6" t="s">
-        <v>119</v>
+        <v>526</v>
       </c>
     </row>
     <row r="416" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6502,10 +6568,10 @@
         <v>516</v>
       </c>
       <c r="B416" s="8" t="s">
-        <v>523</v>
-      </c>
-      <c r="C416" s="6" t="s">
-        <v>119</v>
+        <v>527</v>
+      </c>
+      <c r="C416" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="417" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6516,7 +6582,7 @@
         <v>342</v>
       </c>
       <c r="C417" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="418" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6524,10 +6590,10 @@
         <v>516</v>
       </c>
       <c r="B418" s="8" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="C418" s="6" t="s">
-        <v>119</v>
+        <v>529</v>
       </c>
     </row>
     <row r="419" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6535,10 +6601,10 @@
         <v>516</v>
       </c>
       <c r="B419" s="8" t="s">
-        <v>525</v>
+        <v>530</v>
       </c>
       <c r="C419" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="420" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6546,10 +6612,10 @@
         <v>516</v>
       </c>
       <c r="B420" s="8" t="s">
-        <v>526</v>
+        <v>531</v>
       </c>
       <c r="C420" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="421" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6557,10 +6623,10 @@
         <v>516</v>
       </c>
       <c r="B421" s="8" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="C421" s="6" t="s">
-        <v>119</v>
+        <v>533</v>
       </c>
     </row>
     <row r="422" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6568,10 +6634,10 @@
         <v>516</v>
       </c>
       <c r="B422" s="8" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="C422" s="6" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="423" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6579,10 +6645,10 @@
         <v>516</v>
       </c>
       <c r="B423" s="8" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="C423" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="424" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6590,10 +6656,10 @@
         <v>516</v>
       </c>
       <c r="B424" s="8" t="s">
-        <v>530</v>
+        <v>536</v>
       </c>
       <c r="C424" s="6" t="s">
-        <v>119</v>
+        <v>10</v>
       </c>
     </row>
     <row r="425" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6601,10 +6667,10 @@
         <v>516</v>
       </c>
       <c r="B425" s="8" t="s">
-        <v>531</v>
-      </c>
-      <c r="C425" s="6" t="s">
-        <v>119</v>
+        <v>537</v>
+      </c>
+      <c r="C425" s="9" t="s">
+        <v>538</v>
       </c>
     </row>
     <row r="426" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6612,10 +6678,10 @@
         <v>516</v>
       </c>
       <c r="B426" s="8" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="C426" s="6" t="s">
-        <v>119</v>
+        <v>540</v>
       </c>
     </row>
     <row r="427" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6623,10 +6689,10 @@
         <v>516</v>
       </c>
       <c r="B427" s="8" t="s">
-        <v>533</v>
+        <v>541</v>
       </c>
       <c r="C427" s="6" t="s">
-        <v>119</v>
+        <v>542</v>
       </c>
     </row>
     <row r="428" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6634,10 +6700,10 @@
         <v>516</v>
       </c>
       <c r="B428" s="8" t="s">
-        <v>534</v>
-      </c>
-      <c r="C428" s="6" t="s">
-        <v>119</v>
+        <v>543</v>
+      </c>
+      <c r="C428" s="9" t="s">
+        <v>544</v>
       </c>
     </row>
     <row r="429" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6645,10 +6711,10 @@
         <v>516</v>
       </c>
       <c r="B429" s="8" t="s">
-        <v>535</v>
-      </c>
-      <c r="C429" s="6" t="s">
-        <v>119</v>
+        <v>545</v>
+      </c>
+      <c r="C429" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="430" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6656,54 +6722,54 @@
         <v>516</v>
       </c>
       <c r="B430" s="8" t="s">
-        <v>536</v>
-      </c>
-      <c r="C430" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="431" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>546</v>
+      </c>
+      <c r="C430" s="9" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="431" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B431" s="8" t="s">
-        <v>537</v>
-      </c>
-      <c r="C431" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="432" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>548</v>
+      </c>
+      <c r="C431" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="432" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B432" s="8" t="s">
-        <v>538</v>
-      </c>
-      <c r="C432" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="433" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>549</v>
+      </c>
+      <c r="C432" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="433" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A433" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B433" s="8" t="s">
-        <v>539</v>
+        <v>550</v>
       </c>
       <c r="C433" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="434" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="434" customFormat="false" ht="20.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A434" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B434" s="8" t="s">
-        <v>540</v>
-      </c>
-      <c r="C434" s="6" t="s">
-        <v>119</v>
+        <v>552</v>
+      </c>
+      <c r="C434" s="9" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="435" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6711,43 +6777,43 @@
         <v>516</v>
       </c>
       <c r="B435" s="8" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="C435" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="436" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="436" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A436" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B436" s="8" t="s">
-        <v>542</v>
+        <v>555</v>
       </c>
       <c r="C436" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="437" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="437" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A437" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B437" s="8" t="s">
-        <v>543</v>
-      </c>
-      <c r="C437" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="438" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>556</v>
+      </c>
+      <c r="C437" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="438" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A438" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B438" s="8" t="s">
-        <v>544</v>
-      </c>
-      <c r="C438" s="6" t="s">
-        <v>119</v>
+        <v>557</v>
+      </c>
+      <c r="C438" s="9" t="s">
+        <v>558</v>
       </c>
     </row>
     <row r="439" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6755,21 +6821,21 @@
         <v>516</v>
       </c>
       <c r="B439" s="8" t="s">
-        <v>545</v>
+        <v>559</v>
       </c>
       <c r="C439" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="440" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="440" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B440" s="8" t="s">
-        <v>546</v>
-      </c>
-      <c r="C440" s="6" t="s">
-        <v>119</v>
+        <v>560</v>
+      </c>
+      <c r="C440" s="9" t="s">
+        <v>561</v>
       </c>
     </row>
     <row r="441" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6777,10 +6843,10 @@
         <v>516</v>
       </c>
       <c r="B441" s="8" t="s">
-        <v>547</v>
+        <v>562</v>
       </c>
       <c r="C441" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="442" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6788,54 +6854,54 @@
         <v>516</v>
       </c>
       <c r="B442" s="8" t="s">
-        <v>548</v>
+        <v>563</v>
       </c>
       <c r="C442" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="443" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="443" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B443" s="8" t="s">
-        <v>549</v>
-      </c>
-      <c r="C443" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="444" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>565</v>
+      </c>
+      <c r="C443" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="444" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A444" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B444" s="8" t="s">
-        <v>550</v>
-      </c>
-      <c r="C444" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="445" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>566</v>
+      </c>
+      <c r="C444" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="445" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B445" s="8" t="s">
-        <v>551</v>
+        <v>567</v>
       </c>
       <c r="C445" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="446" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>568</v>
+      </c>
+    </row>
+    <row r="446" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B446" s="8" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
       <c r="C446" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="447" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6843,21 +6909,21 @@
         <v>516</v>
       </c>
       <c r="B447" s="8" t="s">
-        <v>553</v>
+        <v>570</v>
       </c>
       <c r="C447" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="448" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="448" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A448" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B448" s="8" t="s">
-        <v>554</v>
-      </c>
-      <c r="C448" s="6" t="s">
-        <v>119</v>
+        <v>572</v>
+      </c>
+      <c r="C448" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="449" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6865,10 +6931,10 @@
         <v>516</v>
       </c>
       <c r="B449" s="8" t="s">
-        <v>555</v>
+        <v>573</v>
       </c>
       <c r="C449" s="6" t="s">
-        <v>119</v>
+        <v>8</v>
       </c>
     </row>
     <row r="450" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6876,21 +6942,21 @@
         <v>516</v>
       </c>
       <c r="B450" s="8" t="s">
-        <v>556</v>
+        <v>574</v>
       </c>
       <c r="C450" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="451" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="451" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A451" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B451" s="8" t="s">
-        <v>557</v>
-      </c>
-      <c r="C451" s="6" t="s">
-        <v>119</v>
+        <v>575</v>
+      </c>
+      <c r="C451" s="9" t="s">
+        <v>576</v>
       </c>
     </row>
     <row r="452" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6898,43 +6964,43 @@
         <v>516</v>
       </c>
       <c r="B452" s="8" t="s">
-        <v>558</v>
+        <v>577</v>
       </c>
       <c r="C452" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="453" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="453" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A453" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B453" s="8" t="s">
-        <v>559</v>
-      </c>
-      <c r="C453" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="454" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>579</v>
+      </c>
+      <c r="C453" s="9" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="454" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A454" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B454" s="8" t="s">
-        <v>560</v>
-      </c>
-      <c r="C454" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="455" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>581</v>
+      </c>
+      <c r="C454" s="9" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="455" customFormat="false" ht="22.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A455" s="7" t="s">
         <v>516</v>
       </c>
       <c r="B455" s="8" t="s">
-        <v>561</v>
-      </c>
-      <c r="C455" s="6" t="s">
-        <v>119</v>
+        <v>583</v>
+      </c>
+      <c r="C455" s="9" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="456" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6942,7 +7008,7 @@
         <v>516</v>
       </c>
       <c r="B456" s="8" t="s">
-        <v>562</v>
+        <v>584</v>
       </c>
       <c r="C456" s="6" t="s">
         <v>119</v>
@@ -6953,7 +7019,7 @@
         <v>516</v>
       </c>
       <c r="B457" s="8" t="s">
-        <v>563</v>
+        <v>585</v>
       </c>
       <c r="C457" s="6" t="s">
         <v>119</v>
@@ -6964,7 +7030,7 @@
         <v>516</v>
       </c>
       <c r="B458" s="8" t="s">
-        <v>564</v>
+        <v>586</v>
       </c>
       <c r="C458" s="6" t="s">
         <v>119</v>
@@ -6975,7 +7041,7 @@
         <v>516</v>
       </c>
       <c r="B459" s="8" t="s">
-        <v>565</v>
+        <v>587</v>
       </c>
       <c r="C459" s="6" t="s">
         <v>119</v>
@@ -6986,7 +7052,7 @@
         <v>516</v>
       </c>
       <c r="B460" s="8" t="s">
-        <v>566</v>
+        <v>588</v>
       </c>
       <c r="C460" s="6" t="s">
         <v>119</v>
@@ -6997,7 +7063,7 @@
         <v>516</v>
       </c>
       <c r="B461" s="8" t="s">
-        <v>567</v>
+        <v>589</v>
       </c>
       <c r="C461" s="6" t="s">
         <v>119</v>
@@ -7008,7 +7074,7 @@
         <v>516</v>
       </c>
       <c r="B462" s="8" t="s">
-        <v>568</v>
+        <v>590</v>
       </c>
       <c r="C462" s="6" t="s">
         <v>119</v>
@@ -7019,7 +7085,7 @@
         <v>516</v>
       </c>
       <c r="B463" s="8" t="s">
-        <v>569</v>
+        <v>591</v>
       </c>
       <c r="C463" s="6" t="s">
         <v>119</v>
@@ -7030,7 +7096,7 @@
         <v>516</v>
       </c>
       <c r="B464" s="8" t="s">
-        <v>570</v>
+        <v>592</v>
       </c>
       <c r="C464" s="6" t="s">
         <v>119</v>
@@ -7041,7 +7107,7 @@
         <v>516</v>
       </c>
       <c r="B465" s="8" t="s">
-        <v>571</v>
+        <v>593</v>
       </c>
       <c r="C465" s="6" t="s">
         <v>119</v>
@@ -7052,7 +7118,7 @@
         <v>516</v>
       </c>
       <c r="B466" s="8" t="s">
-        <v>572</v>
+        <v>594</v>
       </c>
       <c r="C466" s="6" t="s">
         <v>119</v>
@@ -7063,7 +7129,7 @@
         <v>516</v>
       </c>
       <c r="B467" s="8" t="s">
-        <v>573</v>
+        <v>595</v>
       </c>
       <c r="C467" s="6" t="s">
         <v>119</v>
@@ -7074,7 +7140,7 @@
         <v>516</v>
       </c>
       <c r="B468" s="8" t="s">
-        <v>574</v>
+        <v>596</v>
       </c>
       <c r="C468" s="6" t="s">
         <v>119</v>
@@ -7085,7 +7151,7 @@
         <v>516</v>
       </c>
       <c r="B469" s="8" t="s">
-        <v>575</v>
+        <v>597</v>
       </c>
       <c r="C469" s="6" t="s">
         <v>119</v>
@@ -7104,10 +7170,10 @@
     </row>
     <row r="472" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A472" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B472" s="8" t="s">
-        <v>577</v>
+        <v>599</v>
       </c>
       <c r="C472" s="6" t="s">
         <v>8</v>
@@ -7115,98 +7181,98 @@
     </row>
     <row r="473" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A473" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B473" s="8" t="s">
-        <v>578</v>
+        <v>600</v>
       </c>
       <c r="C473" s="6" t="s">
-        <v>579</v>
+        <v>601</v>
       </c>
     </row>
     <row r="474" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A474" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B474" s="8" t="s">
-        <v>580</v>
+        <v>602</v>
       </c>
       <c r="C474" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="475" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="475" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A475" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B475" s="8" t="s">
-        <v>581</v>
+        <v>603</v>
       </c>
       <c r="C475" s="9" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="476" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="476" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A476" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B476" s="8" t="s">
-        <v>583</v>
+        <v>605</v>
       </c>
       <c r="C476" s="9" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="477" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A477" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B477" s="8" t="s">
-        <v>585</v>
+        <v>607</v>
       </c>
       <c r="C477" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="478" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="478" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A478" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B478" s="8" t="s">
-        <v>586</v>
+        <v>608</v>
       </c>
       <c r="C478" s="9" t="s">
-        <v>587</v>
-      </c>
-    </row>
-    <row r="479" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A479" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B479" s="8" t="s">
-        <v>588</v>
+        <v>610</v>
       </c>
       <c r="C479" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="480" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="480" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A480" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B480" s="8" t="s">
-        <v>589</v>
+        <v>611</v>
       </c>
       <c r="C480" s="9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="481" customFormat="false" ht="19.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="481" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A481" s="7" t="s">
-        <v>576</v>
+        <v>598</v>
       </c>
       <c r="B481" s="8" t="s">
-        <v>590</v>
+        <v>612</v>
       </c>
       <c r="C481" s="9" t="s">
         <v>10</v>
@@ -7615,7 +7681,7 @@
     <hyperlink ref="B433" r:id="rId399" display="Maximum Length Chain of Pairs"/>
     <hyperlink ref="B434" r:id="rId400" display="Maximum size square sub-matrix with all 1s"/>
     <hyperlink ref="B435" r:id="rId401" display="Maximum sum of pairs with specific difference"/>
-    <hyperlink ref="B436" r:id="rId402" display="Min Cost PathProblem"/>
+    <hyperlink ref="B436" r:id="rId402" display="Max Cost PathProblem"/>
     <hyperlink ref="B437" r:id="rId403" display="Maximum difference of zeros and ones in binary string"/>
     <hyperlink ref="B438" r:id="rId404" display="Minimum number of jumps to reach end"/>
     <hyperlink ref="B439" r:id="rId405" display="Minimum cost to fill given weight in a bag"/>

</xml_diff>